<commit_message>
Regenerate 2018 pipeline output after band review corrections
Re-ran all 7 pipeline scripts (0_extract_pipl → 6_create_final_report)
against the corrected 2018 Band Review file.

Results: 119 rows, 306 PIPL, 32 routes, 0 removed
  - 74 banded rows (TotalObserved=1, BandCombo=raw band text)
  - 45 unbanded remainder rows
  - Huguenot Memorial Park pt 3 GPS borrowed from 2024 data

Co-Authored-By: Claude Sonnet 4.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Databases/Database3/Output/2018/db3_2018_FINAL.xlsx
+++ b/Databases/Database3/Output/2018/db3_2018_FINAL.xlsx
@@ -458,7 +458,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R121"/>
+  <dimension ref="A1:R120"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -2253,7 +2253,7 @@
         <v>1</v>
       </c>
       <c r="I26" t="n">
-        <v>1</v>
+        <v>17</v>
       </c>
       <c r="J26" t="inlineStr">
         <is>
@@ -2267,11 +2267,7 @@
       </c>
       <c r="L26" t="inlineStr"/>
       <c r="M26" t="inlineStr"/>
-      <c r="N26" t="inlineStr">
-        <is>
-          <t>0 banded birds then none readable</t>
-        </is>
-      </c>
+      <c r="N26" t="inlineStr"/>
       <c r="O26" t="inlineStr">
         <is>
           <t>Many birds using mudflats to roost and forage in mixed flocks on rising tide</t>
@@ -2298,53 +2294,53 @@
         <v>26</v>
       </c>
       <c r="B27" s="2" t="n">
-        <v>43136</v>
+        <v>43133</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>10:30:00</t>
+          <t>12:11:00</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>50-60F, Medium Wind, No Rain</t>
+          <t>Medium Wind, No Rain</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Big Talbot Island State Park - Spoonbill</t>
+          <t>Buck Beach</t>
         </is>
       </c>
       <c r="F27" t="n">
-        <v>30.50892</v>
+        <v>29.99092</v>
       </c>
       <c r="G27" t="n">
-        <v>-81.4785</v>
+        <v>-85.502</v>
       </c>
       <c r="H27" t="n">
         <v>1</v>
       </c>
       <c r="I27" t="n">
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>Allison Conboy</t>
+          <t>Chris Lipps</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t>Allison.Conboy@dep.state.fl.us</t>
+          <t>clipps@audubon.org</t>
         </is>
       </c>
       <c r="L27" t="inlineStr"/>
       <c r="M27" t="inlineStr"/>
-      <c r="N27" t="inlineStr"/>
-      <c r="O27" t="inlineStr">
-        <is>
-          <t>Many birds using mudflats to roost and forage in mixed flocks on rising tide</t>
-        </is>
-      </c>
+      <c r="N27" t="inlineStr">
+        <is>
+          <t>Of//RB:S//b</t>
+        </is>
+      </c>
+      <c r="O27" t="inlineStr"/>
       <c r="P27" t="inlineStr">
         <is>
           <t>WinterBirdSurvey</t>
@@ -2409,7 +2405,7 @@
       <c r="M28" t="inlineStr"/>
       <c r="N28" t="inlineStr">
         <is>
-          <t>Of//RB:S//b</t>
+          <t>Yf(9C8)//WB:S//bO</t>
         </is>
       </c>
       <c r="O28" t="inlineStr"/>
@@ -2477,7 +2473,7 @@
       <c r="M29" t="inlineStr"/>
       <c r="N29" t="inlineStr">
         <is>
-          <t>Yf(9C8)//WB:S//bO</t>
+          <t>X:X (not banded) 6 total for this point</t>
         </is>
       </c>
       <c r="O29" t="inlineStr"/>
@@ -2529,7 +2525,7 @@
         <v>1</v>
       </c>
       <c r="I30" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="J30" t="inlineStr">
         <is>
@@ -2543,11 +2539,7 @@
       </c>
       <c r="L30" t="inlineStr"/>
       <c r="M30" t="inlineStr"/>
-      <c r="N30" t="inlineStr">
-        <is>
-          <t>X:X (not banded) 6 total for this point</t>
-        </is>
-      </c>
+      <c r="N30" t="inlineStr"/>
       <c r="O30" t="inlineStr"/>
       <c r="P30" t="inlineStr">
         <is>
@@ -2574,44 +2566,48 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>12:11:00</t>
+          <t>11:49:00</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Medium Wind, No Rain</t>
+          <t>60-70F, Calm, No Rain</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Buck Beach</t>
+          <t>Caladesi Island State Park</t>
         </is>
       </c>
       <c r="F31" t="n">
-        <v>29.99092</v>
+        <v>28.05099</v>
       </c>
       <c r="G31" t="n">
-        <v>-85.502</v>
+        <v>-82.8197</v>
       </c>
       <c r="H31" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I31" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>Chris Lipps</t>
+          <t>Frank Brandt, Mike Dyer, Dennis Hunting</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
         <is>
-          <t>clipps@audubon.org</t>
+          <t>fbrandt135@gmail.com michael.dyer@dep.state.fl.us</t>
         </is>
       </c>
       <c r="L31" t="inlineStr"/>
       <c r="M31" t="inlineStr"/>
-      <c r="N31" t="inlineStr"/>
+      <c r="N31" t="inlineStr">
+        <is>
+          <t>LL=FO,G/K RL=_,B</t>
+        </is>
+      </c>
       <c r="O31" t="inlineStr"/>
       <c r="P31" t="inlineStr">
         <is>
@@ -2661,7 +2657,7 @@
         <v>2</v>
       </c>
       <c r="I32" t="n">
-        <v>1</v>
+        <v>27</v>
       </c>
       <c r="J32" t="inlineStr">
         <is>
@@ -2675,11 +2671,7 @@
       </c>
       <c r="L32" t="inlineStr"/>
       <c r="M32" t="inlineStr"/>
-      <c r="N32" t="inlineStr">
-        <is>
-          <t>LL=FO,G/K RL=_,B</t>
-        </is>
-      </c>
+      <c r="N32" t="inlineStr"/>
       <c r="O32" t="inlineStr"/>
       <c r="P32" t="inlineStr">
         <is>
@@ -2702,48 +2694,52 @@
         <v>32</v>
       </c>
       <c r="B33" s="2" t="n">
-        <v>43133</v>
+        <v>43134</v>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>11:49:00</t>
+          <t>08:56:00</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>60-70F, Calm, No Rain</t>
+          <t>60-70F, Medium Wind, No Rain</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Caladesi Island State Park</t>
+          <t>Crandon Park Beach</t>
         </is>
       </c>
       <c r="F33" t="n">
-        <v>28.05099</v>
+        <v>25.70076</v>
       </c>
       <c r="G33" t="n">
-        <v>-82.8197</v>
+        <v>-80.1549</v>
       </c>
       <c r="H33" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I33" t="n">
-        <v>27</v>
+        <v>1</v>
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>Frank Brandt, Mike Dyer, Dennis Hunting</t>
+          <t>Robin Diaz, Miriam Avello</t>
         </is>
       </c>
       <c r="K33" t="inlineStr">
         <is>
-          <t>fbrandt135@gmail.com michael.dyer@dep.state.fl.us</t>
+          <t>rd4birds@bellsouth.net</t>
         </is>
       </c>
       <c r="L33" t="inlineStr"/>
       <c r="M33" t="inlineStr"/>
-      <c r="N33" t="inlineStr"/>
+      <c r="N33" t="inlineStr">
+        <is>
+          <t>bf (missing) S, Y/G: -, G/K (photo; 5th winter)</t>
+        </is>
+      </c>
       <c r="O33" t="inlineStr"/>
       <c r="P33" t="inlineStr">
         <is>
@@ -2809,7 +2805,7 @@
       <c r="M34" t="inlineStr"/>
       <c r="N34" t="inlineStr">
         <is>
-          <t>bf (missing) S, Y/G: -, G/K (photo; 5th winter)</t>
+          <t>Gf (5TH), -: O, - (photo; 3rd winter)</t>
         </is>
       </c>
       <c r="O34" t="inlineStr"/>
@@ -2877,7 +2873,7 @@
       <c r="M35" t="inlineStr"/>
       <c r="N35" t="inlineStr">
         <is>
-          <t>Gf (5TH), -: O, - (photo; 3rd winter)</t>
+          <t>O (green dot), O/Y: S, - (photo; 3rd winter)</t>
         </is>
       </c>
       <c r="O35" t="inlineStr"/>
@@ -2945,7 +2941,7 @@
       <c r="M36" t="inlineStr"/>
       <c r="N36" t="inlineStr">
         <is>
-          <t>O (green dot), O/Y: S, - (photo; 3rd winter)</t>
+          <t>Gf (M9E), -: O, - (photo)</t>
         </is>
       </c>
       <c r="O36" t="inlineStr"/>
@@ -3013,7 +3009,7 @@
       <c r="M37" t="inlineStr"/>
       <c r="N37" t="inlineStr">
         <is>
-          <t>Gf (M9E), -: O, - (photo)</t>
+          <t>Yf (4Y?), -: S, - (photo)</t>
         </is>
       </c>
       <c r="O37" t="inlineStr"/>
@@ -3065,7 +3061,7 @@
         <v>1</v>
       </c>
       <c r="I38" t="n">
-        <v>1</v>
+        <v>27</v>
       </c>
       <c r="J38" t="inlineStr">
         <is>
@@ -3079,11 +3075,7 @@
       </c>
       <c r="L38" t="inlineStr"/>
       <c r="M38" t="inlineStr"/>
-      <c r="N38" t="inlineStr">
-        <is>
-          <t>Yf (4Y?), -: S, - (photo)</t>
-        </is>
-      </c>
+      <c r="N38" t="inlineStr"/>
       <c r="O38" t="inlineStr"/>
       <c r="P38" t="inlineStr">
         <is>
@@ -3124,16 +3116,16 @@
         </is>
       </c>
       <c r="F39" t="n">
-        <v>25.70076</v>
+        <v>25.70171</v>
       </c>
       <c r="G39" t="n">
-        <v>-80.1549</v>
+        <v>-80.1544</v>
       </c>
       <c r="H39" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I39" t="n">
-        <v>27</v>
+        <v>2</v>
       </c>
       <c r="J39" t="inlineStr">
         <is>
@@ -3170,48 +3162,52 @@
         <v>39</v>
       </c>
       <c r="B40" s="2" t="n">
-        <v>43134</v>
+        <v>43137</v>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>08:56:00</t>
+          <t>09:15:00</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>60-70F, Medium Wind, No Rain</t>
+          <t>70-80F, No Rain</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Crandon Park Beach</t>
+          <t>Dunlaton Bridge to Ponce Inlet</t>
         </is>
       </c>
       <c r="F40" t="n">
-        <v>25.70171</v>
+        <v>29.071</v>
       </c>
       <c r="G40" t="n">
-        <v>-80.1544</v>
+        <v>-80.9263</v>
       </c>
       <c r="H40" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="I40" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>Robin Diaz, Miriam Avello</t>
+          <t>M. Brothers, D. Young, J. Winters, B.OKeefe, A. Stevenson</t>
         </is>
       </c>
       <c r="K40" t="inlineStr">
         <is>
-          <t>rd4birds@bellsouth.net</t>
+          <t>mbrothers@volusia.org</t>
         </is>
       </c>
       <c r="L40" t="inlineStr"/>
       <c r="M40" t="inlineStr"/>
-      <c r="N40" t="inlineStr"/>
+      <c r="N40" t="inlineStr">
+        <is>
+          <t>PPI: (UL) FO, (LL) K/O/Y, (UR) S, (LR) Lb (reported to bander);</t>
+        </is>
+      </c>
       <c r="O40" t="inlineStr"/>
       <c r="P40" t="inlineStr">
         <is>
@@ -3277,7 +3273,7 @@
       <c r="M41" t="inlineStr"/>
       <c r="N41" t="inlineStr">
         <is>
-          <t>PPI: (UL) FO, (LL) K/O/Y, (UR) S, (LR) Lb (reported to bander);</t>
+          <t>(UL) S, (LL) Y, (UR) -, (LR) O (reported to bander)</t>
         </is>
       </c>
       <c r="O41" t="inlineStr"/>
@@ -3320,13 +3316,13 @@
         </is>
       </c>
       <c r="F42" t="n">
-        <v>29.071</v>
+        <v>29.07028</v>
       </c>
       <c r="G42" t="n">
-        <v>-80.9263</v>
+        <v>-80.9258</v>
       </c>
       <c r="H42" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="I42" t="n">
         <v>1</v>
@@ -3345,7 +3341,7 @@
       <c r="M42" t="inlineStr"/>
       <c r="N42" t="inlineStr">
         <is>
-          <t>(UL) S, (LL) Y, (UR) -, (LR) O (reported to bander)</t>
+          <t>Band/Flag Code: HY: (UL) S, (LL) -, (UR) FK, (LR) -(reported);</t>
         </is>
       </c>
       <c r="O42" t="inlineStr"/>
@@ -3413,7 +3409,7 @@
       <c r="M43" t="inlineStr"/>
       <c r="N43" t="inlineStr">
         <is>
-          <t>Band/Flag Code: HY: (UL) S, (LL) -, (UR) FK, (LR) -(reported);</t>
+          <t>(UL) S, (LL) B, (UR) FO, (LR) R/Y (reported);</t>
         </is>
       </c>
       <c r="O43" t="inlineStr"/>
@@ -3481,7 +3477,7 @@
       <c r="M44" t="inlineStr"/>
       <c r="N44" t="inlineStr">
         <is>
-          <t>(UL) S, (LL) B, (UR) FO, (LR) R/Y (reported);</t>
+          <t>Band/flag code: LMX: (UL) FG, (LL) -, (UR) B, (LR) - (reported)</t>
         </is>
       </c>
       <c r="O44" t="inlineStr"/>
@@ -3533,7 +3529,7 @@
         <v>7</v>
       </c>
       <c r="I45" t="n">
-        <v>1</v>
+        <v>17</v>
       </c>
       <c r="J45" t="inlineStr">
         <is>
@@ -3547,11 +3543,7 @@
       </c>
       <c r="L45" t="inlineStr"/>
       <c r="M45" t="inlineStr"/>
-      <c r="N45" t="inlineStr">
-        <is>
-          <t>Band/flag code: LMX: (UL) FG, (LL) -, (UR) B, (LR) - (reported)</t>
-        </is>
-      </c>
+      <c r="N45" t="inlineStr"/>
       <c r="O45" t="inlineStr"/>
       <c r="P45" t="inlineStr">
         <is>
@@ -3574,48 +3566,52 @@
         <v>45</v>
       </c>
       <c r="B46" s="2" t="n">
-        <v>43137</v>
+        <v>43136</v>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>09:15:00</t>
+          <t>10:33:00</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>70-80F, No Rain</t>
+          <t>Light Wind, No Rain</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Dunlaton Bridge to Ponce Inlet</t>
+          <t>Eglin AFB - South Restricted</t>
         </is>
       </c>
       <c r="F46" t="n">
-        <v>29.07028</v>
+        <v>29.66549</v>
       </c>
       <c r="G46" t="n">
-        <v>-80.9258</v>
+        <v>-85.3488</v>
       </c>
       <c r="H46" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="I46" t="n">
-        <v>17</v>
+        <v>1</v>
       </c>
       <c r="J46" t="inlineStr">
         <is>
-          <t>M. Brothers, D. Young, J. Winters, B.OKeefe, A. Stevenson</t>
+          <t>Chris Lipps, Molly Tuma</t>
         </is>
       </c>
       <c r="K46" t="inlineStr">
         <is>
-          <t>mbrothers@volusia.org</t>
+          <t>clipps@audubon.org</t>
         </is>
       </c>
       <c r="L46" t="inlineStr"/>
       <c r="M46" t="inlineStr"/>
-      <c r="N46" t="inlineStr"/>
+      <c r="N46" t="inlineStr">
+        <is>
+          <t>S//:Bf(A97)//</t>
+        </is>
+      </c>
       <c r="O46" t="inlineStr"/>
       <c r="P46" t="inlineStr">
         <is>
@@ -3638,53 +3634,57 @@
         <v>46</v>
       </c>
       <c r="B47" s="2" t="n">
-        <v>43136</v>
+        <v>43137</v>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>10:33:00</t>
+          <t>07:50:00</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Light Wind, No Rain</t>
+          <t>60-70F, Medium Wind, No Rain</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Eglin AFB - South Restricted</t>
+          <t>Gulf Islands National Seashore - Perdido Key</t>
         </is>
       </c>
       <c r="F47" t="n">
-        <v>29.66549</v>
+        <v>30.32741</v>
       </c>
       <c r="G47" t="n">
-        <v>-85.3488</v>
+        <v>-87.3137</v>
       </c>
       <c r="H47" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="I47" t="n">
         <v>1</v>
       </c>
       <c r="J47" t="inlineStr">
         <is>
-          <t>Chris Lipps, Molly Tuma</t>
+          <t>Monica Hardin</t>
         </is>
       </c>
       <c r="K47" t="inlineStr">
         <is>
-          <t>clipps@audubon.org</t>
+          <t>hardin6510@gmail.com</t>
         </is>
       </c>
       <c r="L47" t="inlineStr"/>
       <c r="M47" t="inlineStr"/>
       <c r="N47" t="inlineStr">
         <is>
-          <t>S//:Bf(A97)//</t>
-        </is>
-      </c>
-      <c r="O47" t="inlineStr"/>
+          <t>S/LY:bf/LG (bf = light blue flag, no code); reported directly to bander</t>
+        </is>
+      </c>
+      <c r="O47" t="inlineStr">
+        <is>
+          <t>South shore survey</t>
+        </is>
+      </c>
       <c r="P47" t="inlineStr">
         <is>
           <t>WinterBirdSurvey</t>
@@ -3706,55 +3706,55 @@
         <v>47</v>
       </c>
       <c r="B48" s="2" t="n">
-        <v>43137</v>
+        <v>43144</v>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>07:50:00</t>
+          <t>11:40:00</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>60-70F, Medium Wind, No Rain</t>
+          <t>80-90F, Medium Wind, No Rain</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Gulf Islands National Seashore - Perdido Key</t>
+          <t>Highland Beach</t>
         </is>
       </c>
       <c r="F48" t="n">
-        <v>30.32741</v>
+        <v>25.4792</v>
       </c>
       <c r="G48" t="n">
-        <v>-87.3137</v>
+        <v>-81.18680000000001</v>
       </c>
       <c r="H48" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="I48" t="n">
         <v>1</v>
       </c>
       <c r="J48" t="inlineStr">
         <is>
-          <t>Monica Hardin</t>
+          <t>Lori Oberhofer, Britta Muiznieks, John Kipp</t>
         </is>
       </c>
       <c r="K48" t="inlineStr">
         <is>
-          <t>hardin6510@gmail.com</t>
+          <t>lori_oberhofer@nps.gov</t>
         </is>
       </c>
       <c r="L48" t="inlineStr"/>
       <c r="M48" t="inlineStr"/>
       <c r="N48" t="inlineStr">
         <is>
-          <t>S/LY:bf/LG (bf = light blue flag, no code); reported directly to bander</t>
+          <t>YX6, color: green, position: upper left". The "O" is for an orange band on the right leg, position: upper right.</t>
         </is>
       </c>
       <c r="O48" t="inlineStr">
         <is>
-          <t>South shore survey</t>
+          <t>End time was 13:45</t>
         </is>
       </c>
       <c r="P48" t="inlineStr">
@@ -3805,7 +3805,7 @@
         <v>1</v>
       </c>
       <c r="I49" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="J49" t="inlineStr">
         <is>
@@ -3819,11 +3819,7 @@
       </c>
       <c r="L49" t="inlineStr"/>
       <c r="M49" t="inlineStr"/>
-      <c r="N49" t="inlineStr">
-        <is>
-          <t>this is just one says here. One individual. Band/flag code:1) YX6, color: green, position: upper left". The "O" is for an orange band on the right leg, position: upper right.</t>
-        </is>
-      </c>
+      <c r="N49" t="inlineStr"/>
       <c r="O49" t="inlineStr">
         <is>
           <t>End time was 13:45</t>
@@ -3868,16 +3864,16 @@
         </is>
       </c>
       <c r="F50" t="n">
-        <v>25.4792</v>
+        <v>25.50993</v>
       </c>
       <c r="G50" t="n">
-        <v>-81.18680000000001</v>
+        <v>-81.20950000000001</v>
       </c>
       <c r="H50" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I50" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="J50" t="inlineStr">
         <is>
@@ -3918,43 +3914,43 @@
         <v>50</v>
       </c>
       <c r="B51" s="2" t="n">
-        <v>43144</v>
+        <v>43139</v>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>11:40:00</t>
+          <t>09:00:00</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>80-90F, Medium Wind, No Rain</t>
+          <t>50-60F, Light Wind, Light Rain</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Highland Beach</t>
+          <t>Huguenot Memorial Park</t>
         </is>
       </c>
       <c r="F51" t="n">
-        <v>25.50993</v>
+        <v>30.410008</v>
       </c>
       <c r="G51" t="n">
-        <v>-81.20950000000001</v>
+        <v>-81.40774399999999</v>
       </c>
       <c r="H51" t="n">
         <v>3</v>
       </c>
       <c r="I51" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J51" t="inlineStr">
         <is>
-          <t>Lori Oberhofer, Britta Muiznieks, John Kipp</t>
+          <t>Jolie Schlieper, Hailey Garcia</t>
         </is>
       </c>
       <c r="K51" t="inlineStr">
         <is>
-          <t>lori_oberhofer@nps.gov</t>
+          <t>jschlieper@coj.net</t>
         </is>
       </c>
       <c r="L51" t="inlineStr"/>
@@ -3962,7 +3958,7 @@
       <c r="N51" t="inlineStr"/>
       <c r="O51" t="inlineStr">
         <is>
-          <t>End time was 13:45</t>
+          <t>GPS borrowed from 2024 — point 3 had no coordinates in 2018</t>
         </is>
       </c>
       <c r="P51" t="inlineStr">
@@ -3986,53 +3982,49 @@
         <v>51</v>
       </c>
       <c r="B52" s="2" t="n">
-        <v>43139</v>
+        <v>43137</v>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>09:00:00</t>
+          <t>08:25:00</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>50-60F, Light Wind, Light Rain</t>
+          <t>70-80F, Breezy, No Rain</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Huguenot Memorial Park</t>
+          <t>Jupiter &amp; Juno Beach: Jupiter Inlet to northern boundary of John D. MacArthur Beach State Park</t>
         </is>
       </c>
       <c r="F52" t="n">
-        <v>30.410008</v>
+        <v>26.86351</v>
       </c>
       <c r="G52" t="n">
-        <v>-81.40774399999999</v>
+        <v>-80.0475</v>
       </c>
       <c r="H52" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="I52" t="n">
         <v>1</v>
       </c>
       <c r="J52" t="inlineStr">
         <is>
-          <t>Jolie Schlieper, Hailey Garcia</t>
+          <t>Adrienne McCracken &amp; Kim Rigano</t>
         </is>
       </c>
       <c r="K52" t="inlineStr">
         <is>
-          <t>jschlieper@coj.net</t>
+          <t>amccracken@marinelife.org</t>
         </is>
       </c>
       <c r="L52" t="inlineStr"/>
       <c r="M52" t="inlineStr"/>
       <c r="N52" t="inlineStr"/>
-      <c r="O52" t="inlineStr">
-        <is>
-          <t>GPS borrowed from 2024 — point 3 had no coordinates in 2018</t>
-        </is>
-      </c>
+      <c r="O52" t="inlineStr"/>
       <c r="P52" t="inlineStr">
         <is>
           <t>WinterBirdSurvey</t>
@@ -4054,43 +4046,43 @@
         <v>52</v>
       </c>
       <c r="B53" s="2" t="n">
-        <v>43137</v>
+        <v>43135</v>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>08:25:00</t>
+          <t>14:57:00</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>70-80F, Breezy, No Rain</t>
+          <t>80-90F, Medium Wind, No Rain</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Jupiter &amp; Juno Beach: Jupiter Inlet to northern boundary of John D. MacArthur Beach State Park</t>
+          <t>Lake Worth Lagoon</t>
         </is>
       </c>
       <c r="F53" t="n">
-        <v>26.86351</v>
+        <v>26.6232</v>
       </c>
       <c r="G53" t="n">
-        <v>-80.0475</v>
+        <v>-80.0406</v>
       </c>
       <c r="H53" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I53" t="n">
         <v>1</v>
       </c>
       <c r="J53" t="inlineStr">
         <is>
-          <t>Adrienne McCracken &amp; Kim Rigano</t>
+          <t>Ricardo Zambrano</t>
         </is>
       </c>
       <c r="K53" t="inlineStr">
         <is>
-          <t>amccracken@marinelife.org</t>
+          <t>Ricardo.Zambrano@myfwc.com</t>
         </is>
       </c>
       <c r="L53" t="inlineStr"/>
@@ -4118,48 +4110,52 @@
         <v>53</v>
       </c>
       <c r="B54" s="2" t="n">
-        <v>43135</v>
+        <v>43137</v>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>14:57:00</t>
+          <t>10:30:00</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>80-90F, Medium Wind, No Rain</t>
+          <t>50-60F, Calm, No Rain</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Lake Worth Lagoon</t>
+          <t>Lanark Reef</t>
         </is>
       </c>
       <c r="F54" t="n">
-        <v>26.6232</v>
+        <v>29.87753</v>
       </c>
       <c r="G54" t="n">
-        <v>-80.0406</v>
+        <v>-84.5711</v>
       </c>
       <c r="H54" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="I54" t="n">
         <v>1</v>
       </c>
       <c r="J54" t="inlineStr">
         <is>
-          <t>Ricardo Zambrano</t>
+          <t>Laura Garey, Marvin Friel, and Molly Tuma</t>
         </is>
       </c>
       <c r="K54" t="inlineStr">
         <is>
-          <t>Ricardo.Zambrano@myfwc.com</t>
+          <t>lgarey@audubon.org</t>
         </is>
       </c>
       <c r="L54" t="inlineStr"/>
       <c r="M54" t="inlineStr"/>
-      <c r="N54" t="inlineStr"/>
+      <c r="N54" t="inlineStr">
+        <is>
+          <t>S//BK:Bf(C63)//YB</t>
+        </is>
+      </c>
       <c r="O54" t="inlineStr"/>
       <c r="P54" t="inlineStr">
         <is>
@@ -4223,11 +4219,7 @@
       </c>
       <c r="L55" t="inlineStr"/>
       <c r="M55" t="inlineStr"/>
-      <c r="N55" t="inlineStr">
-        <is>
-          <t>S//BK:Bf(C63)//YB</t>
-        </is>
-      </c>
+      <c r="N55" t="inlineStr"/>
       <c r="O55" t="inlineStr"/>
       <c r="P55" t="inlineStr">
         <is>
@@ -4268,13 +4260,13 @@
         </is>
       </c>
       <c r="F56" t="n">
-        <v>29.87753</v>
+        <v>29.87701</v>
       </c>
       <c r="G56" t="n">
-        <v>-84.5711</v>
+        <v>-84.5727</v>
       </c>
       <c r="H56" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="I56" t="n">
         <v>1</v>
@@ -4291,7 +4283,11 @@
       </c>
       <c r="L56" t="inlineStr"/>
       <c r="M56" t="inlineStr"/>
-      <c r="N56" t="inlineStr"/>
+      <c r="N56" t="inlineStr">
+        <is>
+          <t>X//GW:Gf//OO</t>
+        </is>
+      </c>
       <c r="O56" t="inlineStr"/>
       <c r="P56" t="inlineStr">
         <is>
@@ -4357,7 +4353,7 @@
       <c r="M57" t="inlineStr"/>
       <c r="N57" t="inlineStr">
         <is>
-          <t>X//GW:Gf//OO</t>
+          <t>Yf(J87)//RO:S//YB</t>
         </is>
       </c>
       <c r="O57" t="inlineStr"/>
@@ -4425,7 +4421,7 @@
       <c r="M58" t="inlineStr"/>
       <c r="N58" t="inlineStr">
         <is>
-          <t>Yf(J87)//RO:S//YB</t>
+          <t>S//RY:Yf(E60)//YK- all reported to the banders</t>
         </is>
       </c>
       <c r="O58" t="inlineStr"/>
@@ -4477,7 +4473,7 @@
         <v>6</v>
       </c>
       <c r="I59" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J59" t="inlineStr">
         <is>
@@ -4491,11 +4487,7 @@
       </c>
       <c r="L59" t="inlineStr"/>
       <c r="M59" t="inlineStr"/>
-      <c r="N59" t="inlineStr">
-        <is>
-          <t>S//RY:Yf(E60)//YK- all reported to the banders</t>
-        </is>
-      </c>
+      <c r="N59" t="inlineStr"/>
       <c r="O59" t="inlineStr"/>
       <c r="P59" t="inlineStr">
         <is>
@@ -4536,16 +4528,16 @@
         </is>
       </c>
       <c r="F60" t="n">
-        <v>29.87701</v>
+        <v>29.87547</v>
       </c>
       <c r="G60" t="n">
-        <v>-84.5727</v>
+        <v>-84.5741</v>
       </c>
       <c r="H60" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="I60" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J60" t="inlineStr">
         <is>
@@ -4559,7 +4551,11 @@
       </c>
       <c r="L60" t="inlineStr"/>
       <c r="M60" t="inlineStr"/>
-      <c r="N60" t="inlineStr"/>
+      <c r="N60" t="inlineStr">
+        <is>
+          <t>Yf(6H1)//:S//</t>
+        </is>
+      </c>
       <c r="O60" t="inlineStr"/>
       <c r="P60" t="inlineStr">
         <is>
@@ -4609,7 +4605,7 @@
         <v>9</v>
       </c>
       <c r="I61" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J61" t="inlineStr">
         <is>
@@ -4623,11 +4619,7 @@
       </c>
       <c r="L61" t="inlineStr"/>
       <c r="M61" t="inlineStr"/>
-      <c r="N61" t="inlineStr">
-        <is>
-          <t>Yf(6H1)//:S//</t>
-        </is>
-      </c>
+      <c r="N61" t="inlineStr"/>
       <c r="O61" t="inlineStr"/>
       <c r="P61" t="inlineStr">
         <is>
@@ -4668,13 +4660,13 @@
         </is>
       </c>
       <c r="F62" t="n">
-        <v>29.87547</v>
+        <v>29.8754</v>
       </c>
       <c r="G62" t="n">
-        <v>-84.5741</v>
+        <v>-84.57729999999999</v>
       </c>
       <c r="H62" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="I62" t="n">
         <v>2</v>
@@ -4732,16 +4724,16 @@
         </is>
       </c>
       <c r="F63" t="n">
-        <v>29.8754</v>
+        <v>29.87467</v>
       </c>
       <c r="G63" t="n">
-        <v>-84.57729999999999</v>
+        <v>-84.5787</v>
       </c>
       <c r="H63" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="I63" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J63" t="inlineStr">
         <is>
@@ -4755,7 +4747,11 @@
       </c>
       <c r="L63" t="inlineStr"/>
       <c r="M63" t="inlineStr"/>
-      <c r="N63" t="inlineStr"/>
+      <c r="N63" t="inlineStr">
+        <is>
+          <t>Of//OY:S//G</t>
+        </is>
+      </c>
       <c r="O63" t="inlineStr"/>
       <c r="P63" t="inlineStr">
         <is>
@@ -4821,7 +4817,7 @@
       <c r="M64" t="inlineStr"/>
       <c r="N64" t="inlineStr">
         <is>
-          <t>Of//OY:S//G</t>
+          <t>S//YG:Yf(V66)//RO</t>
         </is>
       </c>
       <c r="O64" t="inlineStr"/>
@@ -4873,7 +4869,7 @@
         <v>11</v>
       </c>
       <c r="I65" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J65" t="inlineStr">
         <is>
@@ -4887,11 +4883,7 @@
       </c>
       <c r="L65" t="inlineStr"/>
       <c r="M65" t="inlineStr"/>
-      <c r="N65" t="inlineStr">
-        <is>
-          <t>S//YG:Yf(V66)//RO</t>
-        </is>
-      </c>
+      <c r="N65" t="inlineStr"/>
       <c r="O65" t="inlineStr"/>
       <c r="P65" t="inlineStr">
         <is>
@@ -4918,45 +4910,53 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>10:30:00</t>
+          <t>08:25:00</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>50-60F, Calm, No Rain</t>
+          <t>50-60F, Light Wind, No Rain</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>Lanark Reef</t>
+          <t>Little Talbot Island State Park</t>
         </is>
       </c>
       <c r="F66" t="n">
-        <v>29.87467</v>
+        <v>30.4847</v>
       </c>
       <c r="G66" t="n">
-        <v>-84.5787</v>
+        <v>-81.4153</v>
       </c>
       <c r="H66" t="n">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="I66" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J66" t="inlineStr">
         <is>
-          <t>Laura Garey, Marvin Friel, and Molly Tuma</t>
+          <t>Allison Conboy, Joan Becker, Richard Becker</t>
         </is>
       </c>
       <c r="K66" t="inlineStr">
         <is>
-          <t>lgarey@audubon.org</t>
+          <t>Allison.Conboy@dep.state.fl.us</t>
         </is>
       </c>
       <c r="L66" t="inlineStr"/>
       <c r="M66" t="inlineStr"/>
-      <c r="N66" t="inlineStr"/>
-      <c r="O66" t="inlineStr"/>
+      <c r="N66" t="inlineStr">
+        <is>
+          <t>FO, Lb/R:S,G</t>
+        </is>
+      </c>
+      <c r="O66" t="inlineStr">
+        <is>
+          <t>Sunny, fair weather, rising tide, low at 6:55 a.m.</t>
+        </is>
+      </c>
       <c r="P66" t="inlineStr">
         <is>
           <t>WinterBirdSurvey</t>
@@ -5021,7 +5021,7 @@
       <c r="M67" t="inlineStr"/>
       <c r="N67" t="inlineStr">
         <is>
-          <t>FO, Lb/R:S,G</t>
+          <t>FW[MA], _: S, _</t>
         </is>
       </c>
       <c r="O67" t="inlineStr">
@@ -5093,7 +5093,7 @@
       <c r="M68" t="inlineStr"/>
       <c r="N68" t="inlineStr">
         <is>
-          <t>FW[MA], _: S, _</t>
+          <t>S,_: FW[KC],_</t>
         </is>
       </c>
       <c r="O68" t="inlineStr">
@@ -5165,7 +5165,7 @@
       <c r="M69" t="inlineStr"/>
       <c r="N69" t="inlineStr">
         <is>
-          <t>S,_: FW[KC],_</t>
+          <t>FO,_:G,_</t>
         </is>
       </c>
       <c r="O69" t="inlineStr">
@@ -5237,7 +5237,7 @@
       <c r="M70" t="inlineStr"/>
       <c r="N70" t="inlineStr">
         <is>
-          <t>FO,_:G,_</t>
+          <t>S,B[128]:O(b),B/O</t>
         </is>
       </c>
       <c r="O70" t="inlineStr">
@@ -5309,7 +5309,7 @@
       <c r="M71" t="inlineStr"/>
       <c r="N71" t="inlineStr">
         <is>
-          <t>S,B[128]:O(b),B/O</t>
+          <t>FG[2K6],_:B,_</t>
         </is>
       </c>
       <c r="O71" t="inlineStr">
@@ -5381,7 +5381,7 @@
       <c r="M72" t="inlineStr"/>
       <c r="N72" t="inlineStr">
         <is>
-          <t>FG[2K6],_:B,_</t>
+          <t>FW[VA],_:S,_</t>
         </is>
       </c>
       <c r="O72" t="inlineStr">
@@ -5437,7 +5437,7 @@
         <v>4</v>
       </c>
       <c r="I73" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="J73" t="inlineStr">
         <is>
@@ -5451,11 +5451,7 @@
       </c>
       <c r="L73" t="inlineStr"/>
       <c r="M73" t="inlineStr"/>
-      <c r="N73" t="inlineStr">
-        <is>
-          <t>FW[VA],_:S,_</t>
-        </is>
-      </c>
+      <c r="N73" t="inlineStr"/>
       <c r="O73" t="inlineStr">
         <is>
           <t>Sunny, fair weather, rising tide, low at 6:55 a.m.</t>
@@ -5500,16 +5496,16 @@
         </is>
       </c>
       <c r="F74" t="n">
-        <v>30.4847</v>
+        <v>30.43977</v>
       </c>
       <c r="G74" t="n">
-        <v>-81.4153</v>
+        <v>-81.4081</v>
       </c>
       <c r="H74" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="I74" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="J74" t="inlineStr">
         <is>
@@ -5523,7 +5519,11 @@
       </c>
       <c r="L74" t="inlineStr"/>
       <c r="M74" t="inlineStr"/>
-      <c r="N74" t="inlineStr"/>
+      <c r="N74" t="inlineStr">
+        <is>
+          <t>Banded - FK[UN], _ : S, _</t>
+        </is>
+      </c>
       <c r="O74" t="inlineStr">
         <is>
           <t>Sunny, fair weather, rising tide, low at 6:55 a.m.</t>
@@ -5577,7 +5577,7 @@
         <v>5</v>
       </c>
       <c r="I75" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="J75" t="inlineStr">
         <is>
@@ -5591,11 +5591,7 @@
       </c>
       <c r="L75" t="inlineStr"/>
       <c r="M75" t="inlineStr"/>
-      <c r="N75" t="inlineStr">
-        <is>
-          <t>4 Unbanded, 1) Banded - FK[UN], _ : S, _</t>
-        </is>
-      </c>
+      <c r="N75" t="inlineStr"/>
       <c r="O75" t="inlineStr">
         <is>
           <t>Sunny, fair weather, rising tide, low at 6:55 a.m.</t>
@@ -5640,16 +5636,16 @@
         </is>
       </c>
       <c r="F76" t="n">
-        <v>30.43977</v>
+        <v>30.4329</v>
       </c>
       <c r="G76" t="n">
-        <v>-81.4081</v>
+        <v>-81.407</v>
       </c>
       <c r="H76" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I76" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="J76" t="inlineStr">
         <is>
@@ -5694,49 +5690,45 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>08:25:00</t>
+          <t>07:52:00</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>50-60F, Light Wind, No Rain</t>
+          <t>70-80F, Medium Wind, No Rain</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>Little Talbot Island State Park</t>
+          <t>Long Key State Park</t>
         </is>
       </c>
       <c r="F77" t="n">
-        <v>30.4329</v>
+        <v>24.80786</v>
       </c>
       <c r="G77" t="n">
-        <v>-81.407</v>
+        <v>-80.83499999999999</v>
       </c>
       <c r="H77" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="I77" t="n">
         <v>1</v>
       </c>
       <c r="J77" t="inlineStr">
         <is>
-          <t>Allison Conboy, Joan Becker, Richard Becker</t>
+          <t>Janice Duquesnel, Becky Collins, Mark Lee, Susan Kolterman</t>
         </is>
       </c>
       <c r="K77" t="inlineStr">
         <is>
-          <t>Allison.Conboy@dep.state.fl.us</t>
+          <t>Janice.Duquesnel@dep.state.fl.us</t>
         </is>
       </c>
       <c r="L77" t="inlineStr"/>
       <c r="M77" t="inlineStr"/>
       <c r="N77" t="inlineStr"/>
-      <c r="O77" t="inlineStr">
-        <is>
-          <t>Sunny, fair weather, rising tide, low at 6:55 a.m.</t>
-        </is>
-      </c>
+      <c r="O77" t="inlineStr"/>
       <c r="P77" t="inlineStr">
         <is>
           <t>WinterBirdSurvey</t>
@@ -5776,16 +5768,16 @@
         </is>
       </c>
       <c r="F78" t="n">
-        <v>24.80786</v>
+        <v>24.80772</v>
       </c>
       <c r="G78" t="n">
-        <v>-80.83499999999999</v>
+        <v>-80.8355</v>
       </c>
       <c r="H78" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I78" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="J78" t="inlineStr">
         <is>
@@ -5826,44 +5818,48 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>07:52:00</t>
+          <t>09:20:00</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>70-80F, Medium Wind, No Rain</t>
+          <t>80-90F, Breezy</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>Long Key State Park</t>
+          <t>Martin County IRL</t>
         </is>
       </c>
       <c r="F79" t="n">
-        <v>24.80772</v>
+        <v>27.17168</v>
       </c>
       <c r="G79" t="n">
-        <v>-80.8355</v>
+        <v>-80.1833</v>
       </c>
       <c r="H79" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I79" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="J79" t="inlineStr">
         <is>
-          <t>Janice Duquesnel, Becky Collins, Mark Lee, Susan Kolterman</t>
+          <t>Ricardo Zambrano, Andrea Pereyra, Dan O'Malley</t>
         </is>
       </c>
       <c r="K79" t="inlineStr">
         <is>
-          <t>Janice.Duquesnel@dep.state.fl.us</t>
+          <t>Ricardo.Zambrano@myfwc.com</t>
         </is>
       </c>
       <c r="L79" t="inlineStr"/>
       <c r="M79" t="inlineStr"/>
-      <c r="N79" t="inlineStr"/>
+      <c r="N79" t="inlineStr">
+        <is>
+          <t>Left leg: Orange flag, upper yellow band, lower green band. Right leg: Upper silver USFWS band, lower Yellow band</t>
+        </is>
+      </c>
       <c r="O79" t="inlineStr"/>
       <c r="P79" t="inlineStr">
         <is>
@@ -5927,11 +5923,7 @@
       </c>
       <c r="L80" t="inlineStr"/>
       <c r="M80" t="inlineStr"/>
-      <c r="N80" t="inlineStr">
-        <is>
-          <t>Left leg: Orange flag, upper yellow band, lower green band. Right leg: Upper silver USFWS band, lower Yellow band</t>
-        </is>
-      </c>
+      <c r="N80" t="inlineStr"/>
       <c r="O80" t="inlineStr"/>
       <c r="P80" t="inlineStr">
         <is>
@@ -5954,28 +5946,28 @@
         <v>80</v>
       </c>
       <c r="B81" s="2" t="n">
-        <v>43137</v>
+        <v>43138</v>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>09:20:00</t>
+          <t>09:15:00</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>80-90F, Breezy</t>
+          <t>60-70F, Calm, No Rain</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>Martin County IRL</t>
+          <t>Morgan Bay/Cape Romano</t>
         </is>
       </c>
       <c r="F81" t="n">
-        <v>27.17168</v>
+        <v>25.85589</v>
       </c>
       <c r="G81" t="n">
-        <v>-80.1833</v>
+        <v>-81.68340000000001</v>
       </c>
       <c r="H81" t="n">
         <v>1</v>
@@ -5985,17 +5977,21 @@
       </c>
       <c r="J81" t="inlineStr">
         <is>
-          <t>Ricardo Zambrano, Andrea Pereyra, Dan O'Malley</t>
+          <t>Kim Savides</t>
         </is>
       </c>
       <c r="K81" t="inlineStr">
         <is>
-          <t>Ricardo.Zambrano@myfwc.com</t>
+          <t>kim.savides@gmail.com</t>
         </is>
       </c>
       <c r="L81" t="inlineStr"/>
       <c r="M81" t="inlineStr"/>
-      <c r="N81" t="inlineStr"/>
+      <c r="N81" t="inlineStr">
+        <is>
+          <t>fY(20E),BO:X,Rb continuing bird, will be batch reported at end of season.</t>
+        </is>
+      </c>
       <c r="O81" t="inlineStr"/>
       <c r="P81" t="inlineStr">
         <is>
@@ -6061,7 +6057,7 @@
       <c r="M82" t="inlineStr"/>
       <c r="N82" t="inlineStr">
         <is>
-          <t>fY(20E),BO:X,Rb continuing bird, will be batch reported at end of season.</t>
+          <t>G,-:fG(K5K),- continuing bird, will be batch reported at end of season.</t>
         </is>
       </c>
       <c r="O82" t="inlineStr"/>
@@ -6129,7 +6125,7 @@
       <c r="M83" t="inlineStr"/>
       <c r="N83" t="inlineStr">
         <is>
-          <t>G,-:fG(K5K),- continuing bird, will be batch reported at end of season.</t>
+          <t>X,-:fK(KT),- continuing bird, will be batch reported at end of season.</t>
         </is>
       </c>
       <c r="O83" t="inlineStr"/>
@@ -6197,7 +6193,7 @@
       <c r="M84" t="inlineStr"/>
       <c r="N84" t="inlineStr">
         <is>
-          <t>X,-:fK(KT),- continuing bird, will be batch reported at end of season.</t>
+          <t>X,O/R:O(B.),R(125) reported to Great Lakes Plover coordinators</t>
         </is>
       </c>
       <c r="O84" t="inlineStr"/>
@@ -6249,7 +6245,7 @@
         <v>1</v>
       </c>
       <c r="I85" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="J85" t="inlineStr">
         <is>
@@ -6263,11 +6259,7 @@
       </c>
       <c r="L85" t="inlineStr"/>
       <c r="M85" t="inlineStr"/>
-      <c r="N85" t="inlineStr">
-        <is>
-          <t>X,O/R:O(B.),R(125) reported to Great Lakes Plover coordinators</t>
-        </is>
-      </c>
+      <c r="N85" t="inlineStr"/>
       <c r="O85" t="inlineStr"/>
       <c r="P85" t="inlineStr">
         <is>
@@ -6290,43 +6282,39 @@
         <v>85</v>
       </c>
       <c r="B86" s="2" t="n">
-        <v>43138</v>
+        <v>43139</v>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>09:15:00</t>
-        </is>
-      </c>
-      <c r="D86" t="inlineStr">
-        <is>
-          <t>60-70F, Calm, No Rain</t>
-        </is>
-      </c>
+          <t>08:29:00</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr"/>
       <c r="E86" t="inlineStr">
         <is>
-          <t>Morgan Bay/Cape Romano</t>
+          <t>N. Hutchinson Island (north of John Brooks Beachside Park)</t>
         </is>
       </c>
       <c r="F86" t="n">
-        <v>25.85589</v>
+        <v>27.43161</v>
       </c>
       <c r="G86" t="n">
-        <v>-81.68340000000001</v>
+        <v>-80.27630000000001</v>
       </c>
       <c r="H86" t="n">
         <v>1</v>
       </c>
       <c r="I86" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="J86" t="inlineStr">
         <is>
-          <t>Kim Savides</t>
+          <t>Tim Towles</t>
         </is>
       </c>
       <c r="K86" t="inlineStr">
         <is>
-          <t>kim.savides@gmail.com</t>
+          <t>Tim.Towles@myFWC.com</t>
         </is>
       </c>
       <c r="L86" t="inlineStr"/>
@@ -6368,16 +6356,16 @@
         </is>
       </c>
       <c r="F87" t="n">
-        <v>27.43161</v>
+        <v>27.43255</v>
       </c>
       <c r="G87" t="n">
-        <v>-80.27630000000001</v>
+        <v>-80.27670000000001</v>
       </c>
       <c r="H87" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I87" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J87" t="inlineStr">
         <is>
@@ -6391,7 +6379,11 @@
       </c>
       <c r="L87" t="inlineStr"/>
       <c r="M87" t="inlineStr"/>
-      <c r="N87" t="inlineStr"/>
+      <c r="N87" t="inlineStr">
+        <is>
+          <t>left-- green flag NLP, right-- blue band</t>
+        </is>
+      </c>
       <c r="O87" t="inlineStr"/>
       <c r="P87" t="inlineStr">
         <is>
@@ -6414,46 +6406,50 @@
         <v>87</v>
       </c>
       <c r="B88" s="2" t="n">
-        <v>43139</v>
+        <v>43137</v>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>08:29:00</t>
-        </is>
-      </c>
-      <c r="D88" t="inlineStr"/>
+          <t>13:30:00</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>70-80F, Medium Wind, No Rain</t>
+        </is>
+      </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>N. Hutchinson Island (north of John Brooks Beachside Park)</t>
+          <t>Navarre Beach Sound Side</t>
         </is>
       </c>
       <c r="F88" t="n">
-        <v>27.43255</v>
+        <v>30.3858</v>
       </c>
       <c r="G88" t="n">
-        <v>-80.27670000000001</v>
+        <v>-86.8536</v>
       </c>
       <c r="H88" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I88" t="n">
         <v>1</v>
       </c>
       <c r="J88" t="inlineStr">
         <is>
-          <t>Tim Towles</t>
+          <t>Caroline Stahala</t>
         </is>
       </c>
       <c r="K88" t="inlineStr">
         <is>
-          <t>Tim.Towles@myFWC.com</t>
+          <t>cstahala@audubon.org</t>
         </is>
       </c>
       <c r="L88" t="inlineStr"/>
       <c r="M88" t="inlineStr"/>
       <c r="N88" t="inlineStr">
         <is>
-          <t>left-- green flag NLP, right-- blue band</t>
+          <t>Silver band//white : yellow flag//black</t>
         </is>
       </c>
       <c r="O88" t="inlineStr"/>
@@ -6478,53 +6474,57 @@
         <v>88</v>
       </c>
       <c r="B89" s="2" t="n">
-        <v>43137</v>
+        <v>43134</v>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>13:30:00</t>
+          <t>10:30:00</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>70-80F, Medium Wind, No Rain</t>
+          <t>60-70F, Medium Wind, No Rain</t>
         </is>
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>Navarre Beach Sound Side</t>
+          <t>Outback Key</t>
         </is>
       </c>
       <c r="F89" t="n">
-        <v>30.3858</v>
+        <v>27.6495</v>
       </c>
       <c r="G89" t="n">
-        <v>-86.8536</v>
+        <v>-82.7501</v>
       </c>
       <c r="H89" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I89" t="n">
         <v>1</v>
       </c>
       <c r="J89" t="inlineStr">
         <is>
-          <t>Caroline Stahala</t>
+          <t>P.Plage, M. Parks, E. Plage L. Margeson, D. Margeson</t>
         </is>
       </c>
       <c r="K89" t="inlineStr">
         <is>
-          <t>cstahala@audubon.org</t>
+          <t>peter_plage@fws.gov</t>
         </is>
       </c>
       <c r="L89" t="inlineStr"/>
       <c r="M89" t="inlineStr"/>
       <c r="N89" t="inlineStr">
         <is>
-          <t>Silver band//white : yellow flag//black</t>
-        </is>
-      </c>
-      <c r="O89" t="inlineStr"/>
+          <t>-, O : S, Y-O split band Reported to Great Lakes researchers</t>
+        </is>
+      </c>
+      <c r="O89" t="inlineStr">
+        <is>
+          <t>Revision. Please delete the earlier entry for Outback Key.</t>
+        </is>
+      </c>
       <c r="P89" t="inlineStr">
         <is>
           <t>WinterBirdSurvey</t>
@@ -6573,7 +6573,7 @@
         <v>2</v>
       </c>
       <c r="I90" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="J90" t="inlineStr">
         <is>
@@ -6587,11 +6587,7 @@
       </c>
       <c r="L90" t="inlineStr"/>
       <c r="M90" t="inlineStr"/>
-      <c r="N90" t="inlineStr">
-        <is>
-          <t>-, O : S, Y-O split band Reported to Great Lakes researchers</t>
-        </is>
-      </c>
+      <c r="N90" t="inlineStr"/>
       <c r="O90" t="inlineStr">
         <is>
           <t>Revision. Please delete the earlier entry for Outback Key.</t>
@@ -6622,7 +6618,7 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>10:30:00</t>
+          <t>08:15:00</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
@@ -6632,24 +6628,24 @@
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>Outback Key</t>
+          <t>Shell Key Preserve</t>
         </is>
       </c>
       <c r="F91" t="n">
-        <v>27.6495</v>
+        <v>27.6559</v>
       </c>
       <c r="G91" t="n">
-        <v>-82.7501</v>
+        <v>-82.7393</v>
       </c>
       <c r="H91" t="n">
         <v>2</v>
       </c>
       <c r="I91" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="J91" t="inlineStr">
         <is>
-          <t>P.Plage, M. Parks, E. Plage L. Margeson, D. Margeson</t>
+          <t>Peter Plage, Morgan Parks, Eric Plage, Lorraine Margeson, Don Margeson</t>
         </is>
       </c>
       <c r="K91" t="inlineStr">
@@ -6659,10 +6655,14 @@
       </c>
       <c r="L91" t="inlineStr"/>
       <c r="M91" t="inlineStr"/>
-      <c r="N91" t="inlineStr"/>
+      <c r="N91" t="inlineStr">
+        <is>
+          <t>S, B-O split : O, B Reported to Great Lakes researcher</t>
+        </is>
+      </c>
       <c r="O91" t="inlineStr">
         <is>
-          <t>Revision. Please delete the earlier entry for Outback Key.</t>
+          <t>Surveyed Sand Key spit and nearby flats first at very low tide and returned later to count concentrated birds at mid tide. Totals reflect higher count.</t>
         </is>
       </c>
       <c r="P91" t="inlineStr">
@@ -6727,11 +6727,7 @@
       </c>
       <c r="L92" t="inlineStr"/>
       <c r="M92" t="inlineStr"/>
-      <c r="N92" t="inlineStr">
-        <is>
-          <t>S, B-O split : O, B Reported to Great Lakes researcher</t>
-        </is>
-      </c>
+      <c r="N92" t="inlineStr"/>
       <c r="O92" t="inlineStr">
         <is>
           <t>Surveyed Sand Key spit and nearby flats first at very low tide and returned later to count concentrated birds at mid tide. Totals reflect higher count.</t>
@@ -6776,13 +6772,13 @@
         </is>
       </c>
       <c r="F93" t="n">
-        <v>27.6559</v>
+        <v>27.6501</v>
       </c>
       <c r="G93" t="n">
-        <v>-82.7393</v>
+        <v>-82.7347</v>
       </c>
       <c r="H93" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I93" t="n">
         <v>1</v>
@@ -6799,7 +6795,11 @@
       </c>
       <c r="L93" t="inlineStr"/>
       <c r="M93" t="inlineStr"/>
-      <c r="N93" t="inlineStr"/>
+      <c r="N93" t="inlineStr">
+        <is>
+          <t>S, K : FO, B/Y FTP; Y; FTP, - : -, - reported to Great Lakes area researchers</t>
+        </is>
+      </c>
       <c r="O93" t="inlineStr">
         <is>
           <t>Surveyed Sand Key spit and nearby flats first at very low tide and returned later to count concentrated birds at mid tide. Totals reflect higher count.</t>
@@ -6853,7 +6853,7 @@
         <v>3</v>
       </c>
       <c r="I94" t="n">
-        <v>1</v>
+        <v>14</v>
       </c>
       <c r="J94" t="inlineStr">
         <is>
@@ -6867,11 +6867,7 @@
       </c>
       <c r="L94" t="inlineStr"/>
       <c r="M94" t="inlineStr"/>
-      <c r="N94" t="inlineStr">
-        <is>
-          <t>S, K : FO, B/Y FTP; Y; FTP, - : -, - reported to Great Lakes area researchers</t>
-        </is>
-      </c>
+      <c r="N94" t="inlineStr"/>
       <c r="O94" t="inlineStr">
         <is>
           <t>Surveyed Sand Key spit and nearby flats first at very low tide and returned later to count concentrated birds at mid tide. Totals reflect higher count.</t>
@@ -6898,7 +6894,7 @@
         <v>94</v>
       </c>
       <c r="B95" s="2" t="n">
-        <v>43134</v>
+        <v>43138</v>
       </c>
       <c r="C95" t="inlineStr">
         <is>
@@ -6912,39 +6908,39 @@
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>Shell Key Preserve</t>
+          <t>St Vincent NWR</t>
         </is>
       </c>
       <c r="F95" t="n">
-        <v>27.6501</v>
+        <v>29.63802</v>
       </c>
       <c r="G95" t="n">
-        <v>-82.7347</v>
+        <v>-85.148</v>
       </c>
       <c r="H95" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="I95" t="n">
-        <v>14</v>
+        <v>1</v>
       </c>
       <c r="J95" t="inlineStr">
         <is>
-          <t>Peter Plage, Morgan Parks, Eric Plage, Lorraine Margeson, Don Margeson</t>
+          <t>John Murphy</t>
         </is>
       </c>
       <c r="K95" t="inlineStr">
         <is>
-          <t>peter_plage@fws.gov</t>
+          <t>southmoonunder@mchsi.com</t>
         </is>
       </c>
       <c r="L95" t="inlineStr"/>
       <c r="M95" t="inlineStr"/>
-      <c r="N95" t="inlineStr"/>
-      <c r="O95" t="inlineStr">
-        <is>
-          <t>Surveyed Sand Key spit and nearby flats first at very low tide and returned later to count concentrated birds at mid tide. Totals reflect higher count.</t>
-        </is>
-      </c>
+      <c r="N95" t="inlineStr">
+        <is>
+          <t>S//x:YF(622)//x</t>
+        </is>
+      </c>
+      <c r="O95" t="inlineStr"/>
       <c r="P95" t="inlineStr">
         <is>
           <t>WinterBirdSurvey</t>
@@ -7007,11 +7003,7 @@
       </c>
       <c r="L96" t="inlineStr"/>
       <c r="M96" t="inlineStr"/>
-      <c r="N96" t="inlineStr">
-        <is>
-          <t>S//x:YF(622)//x</t>
-        </is>
-      </c>
+      <c r="N96" t="inlineStr"/>
       <c r="O96" t="inlineStr"/>
       <c r="P96" t="inlineStr">
         <is>
@@ -7038,44 +7030,48 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>08:15:00</t>
+          <t>09:18:00</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>60-70F, Medium Wind, No Rain</t>
+          <t>60-70F, Calm, No Rain</t>
         </is>
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>St Vincent NWR</t>
+          <t>St. George State Park</t>
         </is>
       </c>
       <c r="F97" t="n">
-        <v>29.63802</v>
+        <v>29.71343</v>
       </c>
       <c r="G97" t="n">
-        <v>-85.148</v>
+        <v>-84.7499</v>
       </c>
       <c r="H97" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="I97" t="n">
         <v>1</v>
       </c>
       <c r="J97" t="inlineStr">
         <is>
-          <t>John Murphy</t>
+          <t>Caity Reiland-Smith, Molly Tuma</t>
         </is>
       </c>
       <c r="K97" t="inlineStr">
         <is>
-          <t>southmoonunder@mchsi.com</t>
+          <t>Caity.reiland-smith@myfwc.com</t>
         </is>
       </c>
       <c r="L97" t="inlineStr"/>
       <c r="M97" t="inlineStr"/>
-      <c r="N97" t="inlineStr"/>
+      <c r="N97" t="inlineStr">
+        <is>
+          <t>YF(A41)//WK:S//BO</t>
+        </is>
+      </c>
       <c r="O97" t="inlineStr"/>
       <c r="P97" t="inlineStr">
         <is>
@@ -7116,13 +7112,13 @@
         </is>
       </c>
       <c r="F98" t="n">
-        <v>29.71343</v>
+        <v>29.71624</v>
       </c>
       <c r="G98" t="n">
-        <v>-84.7499</v>
+        <v>-84.7466</v>
       </c>
       <c r="H98" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="I98" t="n">
         <v>1</v>
@@ -7139,11 +7135,7 @@
       </c>
       <c r="L98" t="inlineStr"/>
       <c r="M98" t="inlineStr"/>
-      <c r="N98" t="inlineStr">
-        <is>
-          <t>YF(A41)//WK:S//BO</t>
-        </is>
-      </c>
+      <c r="N98" t="inlineStr"/>
       <c r="O98" t="inlineStr"/>
       <c r="P98" t="inlineStr">
         <is>
@@ -7184,13 +7176,13 @@
         </is>
       </c>
       <c r="F99" t="n">
-        <v>29.71624</v>
+        <v>29.71831</v>
       </c>
       <c r="G99" t="n">
-        <v>-84.7466</v>
+        <v>-84.744</v>
       </c>
       <c r="H99" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I99" t="n">
         <v>1</v>
@@ -7207,7 +7199,11 @@
       </c>
       <c r="L99" t="inlineStr"/>
       <c r="M99" t="inlineStr"/>
-      <c r="N99" t="inlineStr"/>
+      <c r="N99" t="inlineStr">
+        <is>
+          <t>YF(59R)//KO:S//YW</t>
+        </is>
+      </c>
       <c r="O99" t="inlineStr"/>
       <c r="P99" t="inlineStr">
         <is>
@@ -7248,13 +7244,13 @@
         </is>
       </c>
       <c r="F100" t="n">
-        <v>29.71831</v>
+        <v>29.73627</v>
       </c>
       <c r="G100" t="n">
-        <v>-84.744</v>
+        <v>-84.7229</v>
       </c>
       <c r="H100" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="I100" t="n">
         <v>1</v>
@@ -7273,7 +7269,7 @@
       <c r="M100" t="inlineStr"/>
       <c r="N100" t="inlineStr">
         <is>
-          <t>YF(59R)//KO:S//YW</t>
+          <t>S//GR:YF(C00)//WK</t>
         </is>
       </c>
       <c r="O100" t="inlineStr"/>
@@ -7316,13 +7312,13 @@
         </is>
       </c>
       <c r="F101" t="n">
-        <v>29.73627</v>
+        <v>29.7464</v>
       </c>
       <c r="G101" t="n">
-        <v>-84.7229</v>
+        <v>-84.7123</v>
       </c>
       <c r="H101" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="I101" t="n">
         <v>1</v>
@@ -7341,7 +7337,7 @@
       <c r="M101" t="inlineStr"/>
       <c r="N101" t="inlineStr">
         <is>
-          <t>S//GR:YF(C00)//WK</t>
+          <t>YO:GF//WY</t>
         </is>
       </c>
       <c r="O101" t="inlineStr"/>
@@ -7409,7 +7405,7 @@
       <c r="M102" t="inlineStr"/>
       <c r="N102" t="inlineStr">
         <is>
-          <t>YO:GF//WY</t>
+          <t>KF//R:S//YO</t>
         </is>
       </c>
       <c r="O102" t="inlineStr"/>
@@ -7475,11 +7471,7 @@
       </c>
       <c r="L103" t="inlineStr"/>
       <c r="M103" t="inlineStr"/>
-      <c r="N103" t="inlineStr">
-        <is>
-          <t>KF//R:S//YO</t>
-        </is>
-      </c>
+      <c r="N103" t="inlineStr"/>
       <c r="O103" t="inlineStr"/>
       <c r="P103" t="inlineStr">
         <is>
@@ -7502,11 +7494,11 @@
         <v>103</v>
       </c>
       <c r="B104" s="2" t="n">
-        <v>43138</v>
+        <v>43133</v>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>09:18:00</t>
+          <t>10:00:00</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
@@ -7516,29 +7508,29 @@
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t>St. George State Park</t>
+          <t>Three Rooker North Island</t>
         </is>
       </c>
       <c r="F104" t="n">
-        <v>29.7464</v>
+        <v>28.13208</v>
       </c>
       <c r="G104" t="n">
-        <v>-84.7123</v>
+        <v>-82.8282</v>
       </c>
       <c r="H104" t="n">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="I104" t="n">
         <v>1</v>
       </c>
       <c r="J104" t="inlineStr">
         <is>
-          <t>Caity Reiland-Smith, Molly Tuma</t>
+          <t>Dana Kerstein, Wendy Lichty</t>
         </is>
       </c>
       <c r="K104" t="inlineStr">
         <is>
-          <t>Caity.reiland-smith@myfwc.com</t>
+          <t>dana.kerstein@gmail.com</t>
         </is>
       </c>
       <c r="L104" t="inlineStr"/>
@@ -7570,44 +7562,48 @@
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>10:00:00</t>
+          <t>09:30:00</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>60-70F, Calm, No Rain</t>
+          <t>50-60F, Calm, No Rain</t>
         </is>
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t>Three Rooker North Island</t>
+          <t>Three Rooker South Island</t>
         </is>
       </c>
       <c r="F105" t="n">
-        <v>28.13208</v>
+        <v>28.11171</v>
       </c>
       <c r="G105" t="n">
-        <v>-82.8282</v>
+        <v>-82.837</v>
       </c>
       <c r="H105" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I105" t="n">
         <v>1</v>
       </c>
       <c r="J105" t="inlineStr">
         <is>
-          <t>Dana Kerstein, Wendy Lichty</t>
+          <t>Bob Lane, Denise Lane, Jane Mann, Steve Mann</t>
         </is>
       </c>
       <c r="K105" t="inlineStr">
         <is>
-          <t>dana.kerstein@gmail.com</t>
+          <t>Bob Lane ohiomagpie@hotmail.com</t>
         </is>
       </c>
       <c r="L105" t="inlineStr"/>
       <c r="M105" t="inlineStr"/>
-      <c r="N105" t="inlineStr"/>
+      <c r="N105" t="inlineStr">
+        <is>
+          <t>LL=S,Y RL=O,Y</t>
+        </is>
+      </c>
       <c r="O105" t="inlineStr"/>
       <c r="P105" t="inlineStr">
         <is>
@@ -7673,7 +7669,7 @@
       <c r="M106" t="inlineStr"/>
       <c r="N106" t="inlineStr">
         <is>
-          <t>LL=S,Y RL=O,Y</t>
+          <t>LL=Lb,G/R RL=S,K/W</t>
         </is>
       </c>
       <c r="O106" t="inlineStr"/>
@@ -7741,7 +7737,7 @@
       <c r="M107" t="inlineStr"/>
       <c r="N107" t="inlineStr">
         <is>
-          <t>LL=Lb,G/R RL=S,K/W</t>
+          <t>LL=FG,_ RL=S,G/G</t>
         </is>
       </c>
       <c r="O107" t="inlineStr"/>
@@ -7809,7 +7805,7 @@
       <c r="M108" t="inlineStr"/>
       <c r="N108" t="inlineStr">
         <is>
-          <t>LL=FG,_ RL=S,G/G</t>
+          <t>LL=S,_ RL=FK,_</t>
         </is>
       </c>
       <c r="O108" t="inlineStr"/>
@@ -7877,7 +7873,7 @@
       <c r="M109" t="inlineStr"/>
       <c r="N109" t="inlineStr">
         <is>
-          <t>LL=S,_ RL=FK,_</t>
+          <t>LL=FO,Y/Y RL=S,K</t>
         </is>
       </c>
       <c r="O109" t="inlineStr"/>
@@ -7945,7 +7941,7 @@
       <c r="M110" t="inlineStr"/>
       <c r="N110" t="inlineStr">
         <is>
-          <t>LL=FO,Y/Y RL=S,K</t>
+          <t>TY5 LL=FY,_ RL=S,_</t>
         </is>
       </c>
       <c r="O110" t="inlineStr"/>
@@ -8013,7 +8009,7 @@
       <c r="M111" t="inlineStr"/>
       <c r="N111" t="inlineStr">
         <is>
-          <t>TY5 LL=FY,_ RL=S,_</t>
+          <t>LL=FY,B/R RL=S,O/B</t>
         </is>
       </c>
       <c r="O111" t="inlineStr"/>
@@ -8065,7 +8061,7 @@
         <v>2</v>
       </c>
       <c r="I112" t="n">
-        <v>1</v>
+        <v>22</v>
       </c>
       <c r="J112" t="inlineStr">
         <is>
@@ -8079,11 +8075,7 @@
       </c>
       <c r="L112" t="inlineStr"/>
       <c r="M112" t="inlineStr"/>
-      <c r="N112" t="inlineStr">
-        <is>
-          <t>LL=FY,B/R RL=S,O/B</t>
-        </is>
-      </c>
+      <c r="N112" t="inlineStr"/>
       <c r="O112" t="inlineStr"/>
       <c r="P112" t="inlineStr">
         <is>
@@ -8110,45 +8102,53 @@
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>09:30:00</t>
+          <t>08:28:00</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>50-60F, Calm, No Rain</t>
+          <t>50-60F, Breezy, No Rain</t>
         </is>
       </c>
       <c r="E113" t="inlineStr">
         <is>
-          <t>Three Rooker South Island</t>
+          <t>Tyndall Shell</t>
         </is>
       </c>
       <c r="F113" t="n">
-        <v>28.11171</v>
+        <v>30.06609</v>
       </c>
       <c r="G113" t="n">
-        <v>-82.837</v>
+        <v>-85.6161</v>
       </c>
       <c r="H113" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I113" t="n">
-        <v>22</v>
+        <v>1</v>
       </c>
       <c r="J113" t="inlineStr">
         <is>
-          <t>Bob Lane, Denise Lane, Jane Mann, Steve Mann</t>
+          <t>Marvin Friel</t>
         </is>
       </c>
       <c r="K113" t="inlineStr">
         <is>
-          <t>Bob Lane ohiomagpie@hotmail.com</t>
+          <t>marvin.friel@myfwc.com</t>
         </is>
       </c>
       <c r="L113" t="inlineStr"/>
       <c r="M113" t="inlineStr"/>
-      <c r="N113" t="inlineStr"/>
-      <c r="O113" t="inlineStr"/>
+      <c r="N113" t="inlineStr">
+        <is>
+          <t>Of//BB:S//Y</t>
+        </is>
+      </c>
+      <c r="O113" t="inlineStr">
+        <is>
+          <t>End time: 1154</t>
+        </is>
+      </c>
       <c r="P113" t="inlineStr">
         <is>
           <t>WinterBirdSurvey</t>
@@ -8213,7 +8213,7 @@
       <c r="M114" t="inlineStr"/>
       <c r="N114" t="inlineStr">
         <is>
-          <t>Of//BB:S//Y</t>
+          <t>O(blue dot)//Y:S//Y/O</t>
         </is>
       </c>
       <c r="O114" t="inlineStr">
@@ -8285,7 +8285,7 @@
       <c r="M115" t="inlineStr"/>
       <c r="N115" t="inlineStr">
         <is>
-          <t>O(blue dot)//Y:S//Y/O</t>
+          <t>O//b:S//(missing band light blue, LR )</t>
         </is>
       </c>
       <c r="O115" t="inlineStr">
@@ -8357,7 +8357,7 @@
       <c r="M116" t="inlineStr"/>
       <c r="N116" t="inlineStr">
         <is>
-          <t>O//b:S//(missing band light blue, LR )</t>
+          <t>S//KY:Yf(H67)//W (missing band Red, LR)</t>
         </is>
       </c>
       <c r="O116" t="inlineStr">
@@ -8427,11 +8427,7 @@
       </c>
       <c r="L117" t="inlineStr"/>
       <c r="M117" t="inlineStr"/>
-      <c r="N117" t="inlineStr">
-        <is>
-          <t>S//KY:Yf(H67)//W (missing band Red, LR)</t>
-        </is>
-      </c>
+      <c r="N117" t="inlineStr"/>
       <c r="O117" t="inlineStr">
         <is>
           <t>End time: 1154</t>
@@ -8476,13 +8472,13 @@
         </is>
       </c>
       <c r="F118" t="n">
-        <v>30.06609</v>
+        <v>30.08727</v>
       </c>
       <c r="G118" t="n">
-        <v>-85.6161</v>
+        <v>-85.6602</v>
       </c>
       <c r="H118" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="I118" t="n">
         <v>1</v>
@@ -8499,7 +8495,11 @@
       </c>
       <c r="L118" t="inlineStr"/>
       <c r="M118" t="inlineStr"/>
-      <c r="N118" t="inlineStr"/>
+      <c r="N118" t="inlineStr">
+        <is>
+          <t>X//OG:Gf//KY</t>
+        </is>
+      </c>
       <c r="O118" t="inlineStr">
         <is>
           <t>End time: 1154</t>
@@ -8569,7 +8569,7 @@
       <c r="M119" t="inlineStr"/>
       <c r="N119" t="inlineStr">
         <is>
-          <t>X//OG:Gf//KY</t>
+          <t>Yf(82A)//WB:S//OY</t>
         </is>
       </c>
       <c r="O119" t="inlineStr">
@@ -8598,55 +8598,51 @@
         <v>119</v>
       </c>
       <c r="B120" s="2" t="n">
-        <v>43133</v>
+        <v>43137</v>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>08:28:00</t>
+          <t>07:00:00</t>
         </is>
       </c>
       <c r="D120" t="inlineStr">
         <is>
-          <t>50-60F, Breezy, No Rain</t>
+          <t>60-70F, Medium Wind, No Rain</t>
         </is>
       </c>
       <c r="E120" t="inlineStr">
         <is>
-          <t>Tyndall Shell</t>
+          <t>Volusia County Atlantic Coast, Flagler County Line to north side of Ponce Inlet</t>
         </is>
       </c>
       <c r="F120" t="n">
-        <v>30.08727</v>
+        <v>29.30722</v>
       </c>
       <c r="G120" t="n">
-        <v>-85.6602</v>
+        <v>-81.0467</v>
       </c>
       <c r="H120" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="I120" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J120" t="inlineStr">
         <is>
-          <t>Marvin Friel</t>
+          <t>David Hartgrove, Rachel Ramsey, Joan Tague</t>
         </is>
       </c>
       <c r="K120" t="inlineStr">
         <is>
-          <t>marvin.friel@myfwc.com</t>
+          <t>birdman9@earthlink.net</t>
         </is>
       </c>
       <c r="L120" t="inlineStr"/>
       <c r="M120" t="inlineStr"/>
-      <c r="N120" t="inlineStr">
-        <is>
-          <t>Yf(82A)//WB:S//OY</t>
-        </is>
-      </c>
+      <c r="N120" t="inlineStr"/>
       <c r="O120" t="inlineStr">
         <is>
-          <t>End time: 1154</t>
+          <t>Disappointed that we saw no Red Knots. Surprised by the first ever American Avocets I've ever seen at the ocean shoreline.</t>
         </is>
       </c>
       <c r="P120" t="inlineStr">
@@ -8660,74 +8656,6 @@
         </is>
       </c>
       <c r="R120" t="inlineStr">
-        <is>
-          <t>Sheet1</t>
-        </is>
-      </c>
-    </row>
-    <row r="121">
-      <c r="A121" t="n">
-        <v>120</v>
-      </c>
-      <c r="B121" s="2" t="n">
-        <v>43137</v>
-      </c>
-      <c r="C121" t="inlineStr">
-        <is>
-          <t>07:00:00</t>
-        </is>
-      </c>
-      <c r="D121" t="inlineStr">
-        <is>
-          <t>60-70F, Medium Wind, No Rain</t>
-        </is>
-      </c>
-      <c r="E121" t="inlineStr">
-        <is>
-          <t>Volusia County Atlantic Coast, Flagler County Line to north side of Ponce Inlet</t>
-        </is>
-      </c>
-      <c r="F121" t="n">
-        <v>29.30722</v>
-      </c>
-      <c r="G121" t="n">
-        <v>-81.0467</v>
-      </c>
-      <c r="H121" t="n">
-        <v>6</v>
-      </c>
-      <c r="I121" t="n">
-        <v>2</v>
-      </c>
-      <c r="J121" t="inlineStr">
-        <is>
-          <t>David Hartgrove, Rachel Ramsey, Joan Tague</t>
-        </is>
-      </c>
-      <c r="K121" t="inlineStr">
-        <is>
-          <t>birdman9@earthlink.net</t>
-        </is>
-      </c>
-      <c r="L121" t="inlineStr"/>
-      <c r="M121" t="inlineStr"/>
-      <c r="N121" t="inlineStr"/>
-      <c r="O121" t="inlineStr">
-        <is>
-          <t>Disappointed that we saw no Red Knots. Surprised by the first ever American Avocets I've ever seen at the ocean shoreline.</t>
-        </is>
-      </c>
-      <c r="P121" t="inlineStr">
-        <is>
-          <t>WinterBirdSurvey</t>
-        </is>
-      </c>
-      <c r="Q121" t="inlineStr">
-        <is>
-          <t>Winter Birds 2018 Band Review.xlsx</t>
-        </is>
-      </c>
-      <c r="R121" t="inlineStr">
         <is>
           <t>Sheet1</t>
         </is>
@@ -8801,7 +8729,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-04-26 20:24</t>
+          <t>2026-05-16 17:39</t>
         </is>
       </c>
     </row>
@@ -8856,7 +8784,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>120</v>
+        <v>119</v>
       </c>
     </row>
     <row r="8">
@@ -8898,7 +8826,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>120</v>
+        <v>119</v>
       </c>
     </row>
     <row r="12">

</xml_diff>

<commit_message>
Add 2018–2019 pipeline outputs and biologist review data
Pipeline outputs:
- 2018 FINAL: 118 rows, 306 PIPL, 74 banded — biologist corrections applied
  (prose descriptions translated to standard notation, unreadable cells → unbanded)
- 2019 FINAL: 109 rows, 314 PIPL, 44 banded, 1 removed (New Smyrna duplicate)
  (6 points overridden to unbanded, band formatting normalised)

Review data:
- Database3BandReview/ — AI-structured band cells for 2018–2024
- Database3AIBandReview/ — AI-reviewed 2019 band cells (work in progress)
- Database3BiologistReview/ — Biologist review workbooks:
    Biologist_Band_Review_2018-2024.xlsx (blank template sent to biologists)
    Biologist_Band_Review_Completed_2018-2019.xlsx (completed by biologists)

Co-Authored-By: Claude Sonnet 4.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Databases/Database3/Output/2018/db3_2018_FINAL.xlsx
+++ b/Databases/Database3/Output/2018/db3_2018_FINAL.xlsx
@@ -458,7 +458,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R120"/>
+  <dimension ref="A1:R119"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -474,7 +474,7 @@
     <col width="50" customWidth="1" min="11" max="11"/>
     <col width="12" customWidth="1" min="12" max="12"/>
     <col width="13" customWidth="1" min="13" max="13"/>
-    <col width="50" customWidth="1" min="14" max="14"/>
+    <col width="40" customWidth="1" min="14" max="14"/>
     <col width="50" customWidth="1" min="15" max="15"/>
     <col width="20" customWidth="1" min="16" max="16"/>
     <col width="38" customWidth="1" min="17" max="17"/>
@@ -2457,7 +2457,7 @@
         <v>1</v>
       </c>
       <c r="I29" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="J29" t="inlineStr">
         <is>
@@ -2471,11 +2471,7 @@
       </c>
       <c r="L29" t="inlineStr"/>
       <c r="M29" t="inlineStr"/>
-      <c r="N29" t="inlineStr">
-        <is>
-          <t>X:X (not banded) 6 total for this point</t>
-        </is>
-      </c>
+      <c r="N29" t="inlineStr"/>
       <c r="O29" t="inlineStr"/>
       <c r="P29" t="inlineStr">
         <is>
@@ -2502,44 +2498,48 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>12:11:00</t>
+          <t>11:49:00</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Medium Wind, No Rain</t>
+          <t>60-70F, Calm, No Rain</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Buck Beach</t>
+          <t>Caladesi Island State Park</t>
         </is>
       </c>
       <c r="F30" t="n">
-        <v>29.99092</v>
+        <v>28.05099</v>
       </c>
       <c r="G30" t="n">
-        <v>-85.502</v>
+        <v>-82.8197</v>
       </c>
       <c r="H30" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I30" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>Chris Lipps</t>
+          <t>Frank Brandt, Mike Dyer, Dennis Hunting</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>clipps@audubon.org</t>
+          <t>fbrandt135@gmail.com michael.dyer@dep.state.fl.us</t>
         </is>
       </c>
       <c r="L30" t="inlineStr"/>
       <c r="M30" t="inlineStr"/>
-      <c r="N30" t="inlineStr"/>
+      <c r="N30" t="inlineStr">
+        <is>
+          <t>LL=FO,G/K RL=_,B</t>
+        </is>
+      </c>
       <c r="O30" t="inlineStr"/>
       <c r="P30" t="inlineStr">
         <is>
@@ -2589,7 +2589,7 @@
         <v>2</v>
       </c>
       <c r="I31" t="n">
-        <v>1</v>
+        <v>27</v>
       </c>
       <c r="J31" t="inlineStr">
         <is>
@@ -2603,11 +2603,7 @@
       </c>
       <c r="L31" t="inlineStr"/>
       <c r="M31" t="inlineStr"/>
-      <c r="N31" t="inlineStr">
-        <is>
-          <t>LL=FO,G/K RL=_,B</t>
-        </is>
-      </c>
+      <c r="N31" t="inlineStr"/>
       <c r="O31" t="inlineStr"/>
       <c r="P31" t="inlineStr">
         <is>
@@ -2630,48 +2626,52 @@
         <v>31</v>
       </c>
       <c r="B32" s="2" t="n">
-        <v>43133</v>
+        <v>43134</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>11:49:00</t>
+          <t>08:56:00</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>60-70F, Calm, No Rain</t>
+          <t>60-70F, Medium Wind, No Rain</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Caladesi Island State Park</t>
+          <t>Crandon Park Beach</t>
         </is>
       </c>
       <c r="F32" t="n">
-        <v>28.05099</v>
+        <v>25.70076</v>
       </c>
       <c r="G32" t="n">
-        <v>-82.8197</v>
+        <v>-80.1549</v>
       </c>
       <c r="H32" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I32" t="n">
-        <v>27</v>
+        <v>1</v>
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>Frank Brandt, Mike Dyer, Dennis Hunting</t>
+          <t>Robin Diaz, Miriam Avello</t>
         </is>
       </c>
       <c r="K32" t="inlineStr">
         <is>
-          <t>fbrandt135@gmail.com michael.dyer@dep.state.fl.us</t>
+          <t>rd4birds@bellsouth.net</t>
         </is>
       </c>
       <c r="L32" t="inlineStr"/>
       <c r="M32" t="inlineStr"/>
-      <c r="N32" t="inlineStr"/>
+      <c r="N32" t="inlineStr">
+        <is>
+          <t>bf (missing) S, Y/G: -, G/K</t>
+        </is>
+      </c>
       <c r="O32" t="inlineStr"/>
       <c r="P32" t="inlineStr">
         <is>
@@ -2737,7 +2737,7 @@
       <c r="M33" t="inlineStr"/>
       <c r="N33" t="inlineStr">
         <is>
-          <t>bf (missing) S, Y/G: -, G/K (photo; 5th winter)</t>
+          <t>Gf (5TH), -: O, -</t>
         </is>
       </c>
       <c r="O33" t="inlineStr"/>
@@ -2805,7 +2805,7 @@
       <c r="M34" t="inlineStr"/>
       <c r="N34" t="inlineStr">
         <is>
-          <t>Gf (5TH), -: O, - (photo; 3rd winter)</t>
+          <t>O (green dot), O/Y: S, -</t>
         </is>
       </c>
       <c r="O34" t="inlineStr"/>
@@ -2873,7 +2873,7 @@
       <c r="M35" t="inlineStr"/>
       <c r="N35" t="inlineStr">
         <is>
-          <t>O (green dot), O/Y: S, - (photo; 3rd winter)</t>
+          <t>Gf (M9E), -: O, -</t>
         </is>
       </c>
       <c r="O35" t="inlineStr"/>
@@ -2941,7 +2941,7 @@
       <c r="M36" t="inlineStr"/>
       <c r="N36" t="inlineStr">
         <is>
-          <t>Gf (M9E), -: O, - (photo)</t>
+          <t>Yf (4Y?), -: S, -</t>
         </is>
       </c>
       <c r="O36" t="inlineStr"/>
@@ -2993,7 +2993,7 @@
         <v>1</v>
       </c>
       <c r="I37" t="n">
-        <v>1</v>
+        <v>27</v>
       </c>
       <c r="J37" t="inlineStr">
         <is>
@@ -3007,11 +3007,7 @@
       </c>
       <c r="L37" t="inlineStr"/>
       <c r="M37" t="inlineStr"/>
-      <c r="N37" t="inlineStr">
-        <is>
-          <t>Yf (4Y?), -: S, - (photo)</t>
-        </is>
-      </c>
+      <c r="N37" t="inlineStr"/>
       <c r="O37" t="inlineStr"/>
       <c r="P37" t="inlineStr">
         <is>
@@ -3052,16 +3048,16 @@
         </is>
       </c>
       <c r="F38" t="n">
-        <v>25.70076</v>
+        <v>25.70171</v>
       </c>
       <c r="G38" t="n">
-        <v>-80.1549</v>
+        <v>-80.1544</v>
       </c>
       <c r="H38" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I38" t="n">
-        <v>27</v>
+        <v>2</v>
       </c>
       <c r="J38" t="inlineStr">
         <is>
@@ -3098,48 +3094,52 @@
         <v>38</v>
       </c>
       <c r="B39" s="2" t="n">
-        <v>43134</v>
+        <v>43137</v>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>08:56:00</t>
+          <t>09:15:00</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>60-70F, Medium Wind, No Rain</t>
+          <t>70-80F, No Rain</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Crandon Park Beach</t>
+          <t>Dunlaton Bridge to Ponce Inlet</t>
         </is>
       </c>
       <c r="F39" t="n">
-        <v>25.70171</v>
+        <v>29.071</v>
       </c>
       <c r="G39" t="n">
-        <v>-80.1544</v>
+        <v>-80.9263</v>
       </c>
       <c r="H39" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="I39" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>Robin Diaz, Miriam Avello</t>
+          <t>M. Brothers, D. Young, J. Winters, B.OKeefe, A. Stevenson</t>
         </is>
       </c>
       <c r="K39" t="inlineStr">
         <is>
-          <t>rd4birds@bellsouth.net</t>
+          <t>mbrothers@volusia.org</t>
         </is>
       </c>
       <c r="L39" t="inlineStr"/>
       <c r="M39" t="inlineStr"/>
-      <c r="N39" t="inlineStr"/>
+      <c r="N39" t="inlineStr">
+        <is>
+          <t>(UL) FO, (LL) K/O/Y, (UR) S, (LR) Lb</t>
+        </is>
+      </c>
       <c r="O39" t="inlineStr"/>
       <c r="P39" t="inlineStr">
         <is>
@@ -3205,7 +3205,7 @@
       <c r="M40" t="inlineStr"/>
       <c r="N40" t="inlineStr">
         <is>
-          <t>PPI: (UL) FO, (LL) K/O/Y, (UR) S, (LR) Lb (reported to bander);</t>
+          <t>(UL) S, (LL) Y, (UR) -, (LR) O</t>
         </is>
       </c>
       <c r="O40" t="inlineStr"/>
@@ -3248,13 +3248,13 @@
         </is>
       </c>
       <c r="F41" t="n">
-        <v>29.071</v>
+        <v>29.07028</v>
       </c>
       <c r="G41" t="n">
-        <v>-80.9263</v>
+        <v>-80.9258</v>
       </c>
       <c r="H41" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="I41" t="n">
         <v>1</v>
@@ -3273,7 +3273,7 @@
       <c r="M41" t="inlineStr"/>
       <c r="N41" t="inlineStr">
         <is>
-          <t>(UL) S, (LL) Y, (UR) -, (LR) O (reported to bander)</t>
+          <t>(UL) S, (LL) -, (UR) FK, (LR) ;</t>
         </is>
       </c>
       <c r="O41" t="inlineStr"/>
@@ -3341,7 +3341,7 @@
       <c r="M42" t="inlineStr"/>
       <c r="N42" t="inlineStr">
         <is>
-          <t>Band/Flag Code: HY: (UL) S, (LL) -, (UR) FK, (LR) -(reported);</t>
+          <t>(UL) S, (LL) B, (UR) FO, (LR) R/Y;</t>
         </is>
       </c>
       <c r="O42" t="inlineStr"/>
@@ -3409,7 +3409,7 @@
       <c r="M43" t="inlineStr"/>
       <c r="N43" t="inlineStr">
         <is>
-          <t>(UL) S, (LL) B, (UR) FO, (LR) R/Y (reported);</t>
+          <t>LMX: (UL) FG, (LL) -, (UR) B, (LR)</t>
         </is>
       </c>
       <c r="O43" t="inlineStr"/>
@@ -3461,7 +3461,7 @@
         <v>7</v>
       </c>
       <c r="I44" t="n">
-        <v>1</v>
+        <v>17</v>
       </c>
       <c r="J44" t="inlineStr">
         <is>
@@ -3475,11 +3475,7 @@
       </c>
       <c r="L44" t="inlineStr"/>
       <c r="M44" t="inlineStr"/>
-      <c r="N44" t="inlineStr">
-        <is>
-          <t>Band/flag code: LMX: (UL) FG, (LL) -, (UR) B, (LR) - (reported)</t>
-        </is>
-      </c>
+      <c r="N44" t="inlineStr"/>
       <c r="O44" t="inlineStr"/>
       <c r="P44" t="inlineStr">
         <is>
@@ -3502,48 +3498,52 @@
         <v>44</v>
       </c>
       <c r="B45" s="2" t="n">
-        <v>43137</v>
+        <v>43136</v>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>09:15:00</t>
+          <t>10:33:00</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>70-80F, No Rain</t>
+          <t>Light Wind, No Rain</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Dunlaton Bridge to Ponce Inlet</t>
+          <t>Eglin AFB - South Restricted</t>
         </is>
       </c>
       <c r="F45" t="n">
-        <v>29.07028</v>
+        <v>29.66549</v>
       </c>
       <c r="G45" t="n">
-        <v>-80.9258</v>
+        <v>-85.3488</v>
       </c>
       <c r="H45" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="I45" t="n">
-        <v>17</v>
+        <v>1</v>
       </c>
       <c r="J45" t="inlineStr">
         <is>
-          <t>M. Brothers, D. Young, J. Winters, B.OKeefe, A. Stevenson</t>
+          <t>Chris Lipps, Molly Tuma</t>
         </is>
       </c>
       <c r="K45" t="inlineStr">
         <is>
-          <t>mbrothers@volusia.org</t>
+          <t>clipps@audubon.org</t>
         </is>
       </c>
       <c r="L45" t="inlineStr"/>
       <c r="M45" t="inlineStr"/>
-      <c r="N45" t="inlineStr"/>
+      <c r="N45" t="inlineStr">
+        <is>
+          <t>S//:Bf(A97)//</t>
+        </is>
+      </c>
       <c r="O45" t="inlineStr"/>
       <c r="P45" t="inlineStr">
         <is>
@@ -3566,53 +3566,57 @@
         <v>45</v>
       </c>
       <c r="B46" s="2" t="n">
-        <v>43136</v>
+        <v>43137</v>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>10:33:00</t>
+          <t>07:50:00</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Light Wind, No Rain</t>
+          <t>60-70F, Medium Wind, No Rain</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Eglin AFB - South Restricted</t>
+          <t>Gulf Islands National Seashore - Perdido Key</t>
         </is>
       </c>
       <c r="F46" t="n">
-        <v>29.66549</v>
+        <v>30.32741</v>
       </c>
       <c r="G46" t="n">
-        <v>-85.3488</v>
+        <v>-87.3137</v>
       </c>
       <c r="H46" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="I46" t="n">
         <v>1</v>
       </c>
       <c r="J46" t="inlineStr">
         <is>
-          <t>Chris Lipps, Molly Tuma</t>
+          <t>Monica Hardin</t>
         </is>
       </c>
       <c r="K46" t="inlineStr">
         <is>
-          <t>clipps@audubon.org</t>
+          <t>hardin6510@gmail.com</t>
         </is>
       </c>
       <c r="L46" t="inlineStr"/>
       <c r="M46" t="inlineStr"/>
       <c r="N46" t="inlineStr">
         <is>
-          <t>S//:Bf(A97)//</t>
-        </is>
-      </c>
-      <c r="O46" t="inlineStr"/>
+          <t>S/LY:bf/LG</t>
+        </is>
+      </c>
+      <c r="O46" t="inlineStr">
+        <is>
+          <t>South shore survey</t>
+        </is>
+      </c>
       <c r="P46" t="inlineStr">
         <is>
           <t>WinterBirdSurvey</t>
@@ -3634,55 +3638,55 @@
         <v>46</v>
       </c>
       <c r="B47" s="2" t="n">
-        <v>43137</v>
+        <v>43144</v>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>07:50:00</t>
+          <t>11:40:00</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>60-70F, Medium Wind, No Rain</t>
+          <t>80-90F, Medium Wind, No Rain</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Gulf Islands National Seashore - Perdido Key</t>
+          <t>Highland Beach</t>
         </is>
       </c>
       <c r="F47" t="n">
-        <v>30.32741</v>
+        <v>25.4792</v>
       </c>
       <c r="G47" t="n">
-        <v>-87.3137</v>
+        <v>-81.18680000000001</v>
       </c>
       <c r="H47" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="I47" t="n">
         <v>1</v>
       </c>
       <c r="J47" t="inlineStr">
         <is>
-          <t>Monica Hardin</t>
+          <t>Lori Oberhofer, Britta Muiznieks, John Kipp</t>
         </is>
       </c>
       <c r="K47" t="inlineStr">
         <is>
-          <t>hardin6510@gmail.com</t>
+          <t>lori_oberhofer@nps.gov</t>
         </is>
       </c>
       <c r="L47" t="inlineStr"/>
       <c r="M47" t="inlineStr"/>
       <c r="N47" t="inlineStr">
         <is>
-          <t>S/LY:bf/LG (bf = light blue flag, no code); reported directly to bander</t>
+          <t>fg(YX6)/-:O/M</t>
         </is>
       </c>
       <c r="O47" t="inlineStr">
         <is>
-          <t>South shore survey</t>
+          <t>End time was 13:45</t>
         </is>
       </c>
       <c r="P47" t="inlineStr">
@@ -3733,7 +3737,7 @@
         <v>1</v>
       </c>
       <c r="I48" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="J48" t="inlineStr">
         <is>
@@ -3747,11 +3751,7 @@
       </c>
       <c r="L48" t="inlineStr"/>
       <c r="M48" t="inlineStr"/>
-      <c r="N48" t="inlineStr">
-        <is>
-          <t>YX6, color: green, position: upper left". The "O" is for an orange band on the right leg, position: upper right.</t>
-        </is>
-      </c>
+      <c r="N48" t="inlineStr"/>
       <c r="O48" t="inlineStr">
         <is>
           <t>End time was 13:45</t>
@@ -3796,16 +3796,16 @@
         </is>
       </c>
       <c r="F49" t="n">
-        <v>25.4792</v>
+        <v>25.50993</v>
       </c>
       <c r="G49" t="n">
-        <v>-81.18680000000001</v>
+        <v>-81.20950000000001</v>
       </c>
       <c r="H49" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I49" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="J49" t="inlineStr">
         <is>
@@ -3846,53 +3846,49 @@
         <v>49</v>
       </c>
       <c r="B50" s="2" t="n">
-        <v>43144</v>
+        <v>43139</v>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>11:40:00</t>
+          <t>09:00:00</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>80-90F, Medium Wind, No Rain</t>
+          <t>50-60F, Light Wind, Light Rain</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Highland Beach</t>
+          <t>Huguenot Memorial Park</t>
         </is>
       </c>
       <c r="F50" t="n">
-        <v>25.50993</v>
+        <v>30.410008</v>
       </c>
       <c r="G50" t="n">
-        <v>-81.20950000000001</v>
+        <v>-81.40774399999999</v>
       </c>
       <c r="H50" t="n">
         <v>3</v>
       </c>
       <c r="I50" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J50" t="inlineStr">
         <is>
-          <t>Lori Oberhofer, Britta Muiznieks, John Kipp</t>
+          <t>Jolie Schlieper, Hailey Garcia</t>
         </is>
       </c>
       <c r="K50" t="inlineStr">
         <is>
-          <t>lori_oberhofer@nps.gov</t>
+          <t>jschlieper@coj.net</t>
         </is>
       </c>
       <c r="L50" t="inlineStr"/>
       <c r="M50" t="inlineStr"/>
       <c r="N50" t="inlineStr"/>
-      <c r="O50" t="inlineStr">
-        <is>
-          <t>End time was 13:45</t>
-        </is>
-      </c>
+      <c r="O50" t="inlineStr"/>
       <c r="P50" t="inlineStr">
         <is>
           <t>WinterBirdSurvey</t>
@@ -3914,53 +3910,49 @@
         <v>50</v>
       </c>
       <c r="B51" s="2" t="n">
-        <v>43139</v>
+        <v>43137</v>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>09:00:00</t>
+          <t>08:25:00</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>50-60F, Light Wind, Light Rain</t>
+          <t>70-80F, Breezy, No Rain</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Huguenot Memorial Park</t>
+          <t>Jupiter &amp; Juno Beach: Jupiter Inlet to northern boundary of John D. MacArthur Beach State Park</t>
         </is>
       </c>
       <c r="F51" t="n">
-        <v>30.410008</v>
+        <v>26.86351</v>
       </c>
       <c r="G51" t="n">
-        <v>-81.40774399999999</v>
+        <v>-80.0475</v>
       </c>
       <c r="H51" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="I51" t="n">
         <v>1</v>
       </c>
       <c r="J51" t="inlineStr">
         <is>
-          <t>Jolie Schlieper, Hailey Garcia</t>
+          <t>Adrienne McCracken &amp; Kim Rigano</t>
         </is>
       </c>
       <c r="K51" t="inlineStr">
         <is>
-          <t>jschlieper@coj.net</t>
+          <t>amccracken@marinelife.org</t>
         </is>
       </c>
       <c r="L51" t="inlineStr"/>
       <c r="M51" t="inlineStr"/>
       <c r="N51" t="inlineStr"/>
-      <c r="O51" t="inlineStr">
-        <is>
-          <t>GPS borrowed from 2024 — point 3 had no coordinates in 2018</t>
-        </is>
-      </c>
+      <c r="O51" t="inlineStr"/>
       <c r="P51" t="inlineStr">
         <is>
           <t>WinterBirdSurvey</t>
@@ -3982,43 +3974,43 @@
         <v>51</v>
       </c>
       <c r="B52" s="2" t="n">
-        <v>43137</v>
+        <v>43135</v>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>08:25:00</t>
+          <t>14:57:00</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>70-80F, Breezy, No Rain</t>
+          <t>80-90F, Medium Wind, No Rain</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Jupiter &amp; Juno Beach: Jupiter Inlet to northern boundary of John D. MacArthur Beach State Park</t>
+          <t>Lake Worth Lagoon</t>
         </is>
       </c>
       <c r="F52" t="n">
-        <v>26.86351</v>
+        <v>26.6232</v>
       </c>
       <c r="G52" t="n">
-        <v>-80.0475</v>
+        <v>-80.0406</v>
       </c>
       <c r="H52" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I52" t="n">
         <v>1</v>
       </c>
       <c r="J52" t="inlineStr">
         <is>
-          <t>Adrienne McCracken &amp; Kim Rigano</t>
+          <t>Ricardo Zambrano</t>
         </is>
       </c>
       <c r="K52" t="inlineStr">
         <is>
-          <t>amccracken@marinelife.org</t>
+          <t>Ricardo.Zambrano@myfwc.com</t>
         </is>
       </c>
       <c r="L52" t="inlineStr"/>
@@ -4046,48 +4038,52 @@
         <v>52</v>
       </c>
       <c r="B53" s="2" t="n">
-        <v>43135</v>
+        <v>43137</v>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>14:57:00</t>
+          <t>10:30:00</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>80-90F, Medium Wind, No Rain</t>
+          <t>50-60F, Calm, No Rain</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Lake Worth Lagoon</t>
+          <t>Lanark Reef</t>
         </is>
       </c>
       <c r="F53" t="n">
-        <v>26.6232</v>
+        <v>29.87753</v>
       </c>
       <c r="G53" t="n">
-        <v>-80.0406</v>
+        <v>-84.5711</v>
       </c>
       <c r="H53" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="I53" t="n">
         <v>1</v>
       </c>
       <c r="J53" t="inlineStr">
         <is>
-          <t>Ricardo Zambrano</t>
+          <t>Laura Garey, Marvin Friel, and Molly Tuma</t>
         </is>
       </c>
       <c r="K53" t="inlineStr">
         <is>
-          <t>Ricardo.Zambrano@myfwc.com</t>
+          <t>lgarey@audubon.org</t>
         </is>
       </c>
       <c r="L53" t="inlineStr"/>
       <c r="M53" t="inlineStr"/>
-      <c r="N53" t="inlineStr"/>
+      <c r="N53" t="inlineStr">
+        <is>
+          <t>S//BK:Bf(C63)//YB</t>
+        </is>
+      </c>
       <c r="O53" t="inlineStr"/>
       <c r="P53" t="inlineStr">
         <is>
@@ -4151,11 +4147,7 @@
       </c>
       <c r="L54" t="inlineStr"/>
       <c r="M54" t="inlineStr"/>
-      <c r="N54" t="inlineStr">
-        <is>
-          <t>S//BK:Bf(C63)//YB</t>
-        </is>
-      </c>
+      <c r="N54" t="inlineStr"/>
       <c r="O54" t="inlineStr"/>
       <c r="P54" t="inlineStr">
         <is>
@@ -4196,13 +4188,13 @@
         </is>
       </c>
       <c r="F55" t="n">
-        <v>29.87753</v>
+        <v>29.87701</v>
       </c>
       <c r="G55" t="n">
-        <v>-84.5711</v>
+        <v>-84.5727</v>
       </c>
       <c r="H55" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="I55" t="n">
         <v>1</v>
@@ -4219,7 +4211,11 @@
       </c>
       <c r="L55" t="inlineStr"/>
       <c r="M55" t="inlineStr"/>
-      <c r="N55" t="inlineStr"/>
+      <c r="N55" t="inlineStr">
+        <is>
+          <t>X//GW:Gf//OO</t>
+        </is>
+      </c>
       <c r="O55" t="inlineStr"/>
       <c r="P55" t="inlineStr">
         <is>
@@ -4285,7 +4281,7 @@
       <c r="M56" t="inlineStr"/>
       <c r="N56" t="inlineStr">
         <is>
-          <t>X//GW:Gf//OO</t>
+          <t>Yf(J87)//RO:S//YB</t>
         </is>
       </c>
       <c r="O56" t="inlineStr"/>
@@ -4353,7 +4349,7 @@
       <c r="M57" t="inlineStr"/>
       <c r="N57" t="inlineStr">
         <is>
-          <t>Yf(J87)//RO:S//YB</t>
+          <t>S//RY:Yf(E60)//YK</t>
         </is>
       </c>
       <c r="O57" t="inlineStr"/>
@@ -4405,7 +4401,7 @@
         <v>6</v>
       </c>
       <c r="I58" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J58" t="inlineStr">
         <is>
@@ -4419,11 +4415,7 @@
       </c>
       <c r="L58" t="inlineStr"/>
       <c r="M58" t="inlineStr"/>
-      <c r="N58" t="inlineStr">
-        <is>
-          <t>S//RY:Yf(E60)//YK- all reported to the banders</t>
-        </is>
-      </c>
+      <c r="N58" t="inlineStr"/>
       <c r="O58" t="inlineStr"/>
       <c r="P58" t="inlineStr">
         <is>
@@ -4464,16 +4456,16 @@
         </is>
       </c>
       <c r="F59" t="n">
-        <v>29.87701</v>
+        <v>29.87547</v>
       </c>
       <c r="G59" t="n">
-        <v>-84.5727</v>
+        <v>-84.5741</v>
       </c>
       <c r="H59" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="I59" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J59" t="inlineStr">
         <is>
@@ -4487,7 +4479,11 @@
       </c>
       <c r="L59" t="inlineStr"/>
       <c r="M59" t="inlineStr"/>
-      <c r="N59" t="inlineStr"/>
+      <c r="N59" t="inlineStr">
+        <is>
+          <t>Yf(6H1)//:S//</t>
+        </is>
+      </c>
       <c r="O59" t="inlineStr"/>
       <c r="P59" t="inlineStr">
         <is>
@@ -4537,7 +4533,7 @@
         <v>9</v>
       </c>
       <c r="I60" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J60" t="inlineStr">
         <is>
@@ -4551,11 +4547,7 @@
       </c>
       <c r="L60" t="inlineStr"/>
       <c r="M60" t="inlineStr"/>
-      <c r="N60" t="inlineStr">
-        <is>
-          <t>Yf(6H1)//:S//</t>
-        </is>
-      </c>
+      <c r="N60" t="inlineStr"/>
       <c r="O60" t="inlineStr"/>
       <c r="P60" t="inlineStr">
         <is>
@@ -4596,13 +4588,13 @@
         </is>
       </c>
       <c r="F61" t="n">
-        <v>29.87547</v>
+        <v>29.8754</v>
       </c>
       <c r="G61" t="n">
-        <v>-84.5741</v>
+        <v>-84.57729999999999</v>
       </c>
       <c r="H61" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="I61" t="n">
         <v>2</v>
@@ -4660,16 +4652,16 @@
         </is>
       </c>
       <c r="F62" t="n">
-        <v>29.8754</v>
+        <v>29.87467</v>
       </c>
       <c r="G62" t="n">
-        <v>-84.57729999999999</v>
+        <v>-84.5787</v>
       </c>
       <c r="H62" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="I62" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J62" t="inlineStr">
         <is>
@@ -4683,7 +4675,11 @@
       </c>
       <c r="L62" t="inlineStr"/>
       <c r="M62" t="inlineStr"/>
-      <c r="N62" t="inlineStr"/>
+      <c r="N62" t="inlineStr">
+        <is>
+          <t>Of//OY:S//G</t>
+        </is>
+      </c>
       <c r="O62" t="inlineStr"/>
       <c r="P62" t="inlineStr">
         <is>
@@ -4749,7 +4745,7 @@
       <c r="M63" t="inlineStr"/>
       <c r="N63" t="inlineStr">
         <is>
-          <t>Of//OY:S//G</t>
+          <t>S//YG:Yf(V66)//RO</t>
         </is>
       </c>
       <c r="O63" t="inlineStr"/>
@@ -4801,7 +4797,7 @@
         <v>11</v>
       </c>
       <c r="I64" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J64" t="inlineStr">
         <is>
@@ -4815,11 +4811,7 @@
       </c>
       <c r="L64" t="inlineStr"/>
       <c r="M64" t="inlineStr"/>
-      <c r="N64" t="inlineStr">
-        <is>
-          <t>S//YG:Yf(V66)//RO</t>
-        </is>
-      </c>
+      <c r="N64" t="inlineStr"/>
       <c r="O64" t="inlineStr"/>
       <c r="P64" t="inlineStr">
         <is>
@@ -4846,45 +4838,53 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>10:30:00</t>
+          <t>08:25:00</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>50-60F, Calm, No Rain</t>
+          <t>50-60F, Light Wind, No Rain</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>Lanark Reef</t>
+          <t>Little Talbot Island State Park</t>
         </is>
       </c>
       <c r="F65" t="n">
-        <v>29.87467</v>
+        <v>30.4847</v>
       </c>
       <c r="G65" t="n">
-        <v>-84.5787</v>
+        <v>-81.4153</v>
       </c>
       <c r="H65" t="n">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="I65" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J65" t="inlineStr">
         <is>
-          <t>Laura Garey, Marvin Friel, and Molly Tuma</t>
+          <t>Allison Conboy, Joan Becker, Richard Becker</t>
         </is>
       </c>
       <c r="K65" t="inlineStr">
         <is>
-          <t>lgarey@audubon.org</t>
+          <t>Allison.Conboy@dep.state.fl.us</t>
         </is>
       </c>
       <c r="L65" t="inlineStr"/>
       <c r="M65" t="inlineStr"/>
-      <c r="N65" t="inlineStr"/>
-      <c r="O65" t="inlineStr"/>
+      <c r="N65" t="inlineStr">
+        <is>
+          <t>FO, Lb/R:S,G</t>
+        </is>
+      </c>
+      <c r="O65" t="inlineStr">
+        <is>
+          <t>Sunny, fair weather, rising tide, low at 6:55 a.m.</t>
+        </is>
+      </c>
       <c r="P65" t="inlineStr">
         <is>
           <t>WinterBirdSurvey</t>
@@ -4949,7 +4949,7 @@
       <c r="M66" t="inlineStr"/>
       <c r="N66" t="inlineStr">
         <is>
-          <t>FO, Lb/R:S,G</t>
+          <t>FW[MA], _: S, _</t>
         </is>
       </c>
       <c r="O66" t="inlineStr">
@@ -5021,7 +5021,7 @@
       <c r="M67" t="inlineStr"/>
       <c r="N67" t="inlineStr">
         <is>
-          <t>FW[MA], _: S, _</t>
+          <t>S,_: FW[KC],_</t>
         </is>
       </c>
       <c r="O67" t="inlineStr">
@@ -5093,7 +5093,7 @@
       <c r="M68" t="inlineStr"/>
       <c r="N68" t="inlineStr">
         <is>
-          <t>S,_: FW[KC],_</t>
+          <t>FO,_:G,_</t>
         </is>
       </c>
       <c r="O68" t="inlineStr">
@@ -5165,7 +5165,7 @@
       <c r="M69" t="inlineStr"/>
       <c r="N69" t="inlineStr">
         <is>
-          <t>FO,_:G,_</t>
+          <t>S,B[128]:O(b),B/O</t>
         </is>
       </c>
       <c r="O69" t="inlineStr">
@@ -5237,7 +5237,7 @@
       <c r="M70" t="inlineStr"/>
       <c r="N70" t="inlineStr">
         <is>
-          <t>S,B[128]:O(b),B/O</t>
+          <t>FG[2K6],_:B,_</t>
         </is>
       </c>
       <c r="O70" t="inlineStr">
@@ -5309,7 +5309,7 @@
       <c r="M71" t="inlineStr"/>
       <c r="N71" t="inlineStr">
         <is>
-          <t>FG[2K6],_:B,_</t>
+          <t>FW[VA],_:S,_</t>
         </is>
       </c>
       <c r="O71" t="inlineStr">
@@ -5365,7 +5365,7 @@
         <v>4</v>
       </c>
       <c r="I72" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="J72" t="inlineStr">
         <is>
@@ -5379,11 +5379,7 @@
       </c>
       <c r="L72" t="inlineStr"/>
       <c r="M72" t="inlineStr"/>
-      <c r="N72" t="inlineStr">
-        <is>
-          <t>FW[VA],_:S,_</t>
-        </is>
-      </c>
+      <c r="N72" t="inlineStr"/>
       <c r="O72" t="inlineStr">
         <is>
           <t>Sunny, fair weather, rising tide, low at 6:55 a.m.</t>
@@ -5428,16 +5424,16 @@
         </is>
       </c>
       <c r="F73" t="n">
-        <v>30.4847</v>
+        <v>30.43977</v>
       </c>
       <c r="G73" t="n">
-        <v>-81.4153</v>
+        <v>-81.4081</v>
       </c>
       <c r="H73" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="I73" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="J73" t="inlineStr">
         <is>
@@ -5451,7 +5447,11 @@
       </c>
       <c r="L73" t="inlineStr"/>
       <c r="M73" t="inlineStr"/>
-      <c r="N73" t="inlineStr"/>
+      <c r="N73" t="inlineStr">
+        <is>
+          <t>FK[UN], _ : S, _</t>
+        </is>
+      </c>
       <c r="O73" t="inlineStr">
         <is>
           <t>Sunny, fair weather, rising tide, low at 6:55 a.m.</t>
@@ -5505,7 +5505,7 @@
         <v>5</v>
       </c>
       <c r="I74" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="J74" t="inlineStr">
         <is>
@@ -5519,11 +5519,7 @@
       </c>
       <c r="L74" t="inlineStr"/>
       <c r="M74" t="inlineStr"/>
-      <c r="N74" t="inlineStr">
-        <is>
-          <t>Banded - FK[UN], _ : S, _</t>
-        </is>
-      </c>
+      <c r="N74" t="inlineStr"/>
       <c r="O74" t="inlineStr">
         <is>
           <t>Sunny, fair weather, rising tide, low at 6:55 a.m.</t>
@@ -5568,16 +5564,16 @@
         </is>
       </c>
       <c r="F75" t="n">
-        <v>30.43977</v>
+        <v>30.4329</v>
       </c>
       <c r="G75" t="n">
-        <v>-81.4081</v>
+        <v>-81.407</v>
       </c>
       <c r="H75" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I75" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="J75" t="inlineStr">
         <is>
@@ -5622,49 +5618,45 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>08:25:00</t>
+          <t>07:52:00</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>50-60F, Light Wind, No Rain</t>
+          <t>70-80F, Medium Wind, No Rain</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>Little Talbot Island State Park</t>
+          <t>Long Key State Park</t>
         </is>
       </c>
       <c r="F76" t="n">
-        <v>30.4329</v>
+        <v>24.80786</v>
       </c>
       <c r="G76" t="n">
-        <v>-81.407</v>
+        <v>-80.83499999999999</v>
       </c>
       <c r="H76" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="I76" t="n">
         <v>1</v>
       </c>
       <c r="J76" t="inlineStr">
         <is>
-          <t>Allison Conboy, Joan Becker, Richard Becker</t>
+          <t>Janice Duquesnel, Becky Collins, Mark Lee, Susan Kolterman</t>
         </is>
       </c>
       <c r="K76" t="inlineStr">
         <is>
-          <t>Allison.Conboy@dep.state.fl.us</t>
+          <t>Janice.Duquesnel@dep.state.fl.us</t>
         </is>
       </c>
       <c r="L76" t="inlineStr"/>
       <c r="M76" t="inlineStr"/>
       <c r="N76" t="inlineStr"/>
-      <c r="O76" t="inlineStr">
-        <is>
-          <t>Sunny, fair weather, rising tide, low at 6:55 a.m.</t>
-        </is>
-      </c>
+      <c r="O76" t="inlineStr"/>
       <c r="P76" t="inlineStr">
         <is>
           <t>WinterBirdSurvey</t>
@@ -5704,16 +5696,16 @@
         </is>
       </c>
       <c r="F77" t="n">
-        <v>24.80786</v>
+        <v>24.80772</v>
       </c>
       <c r="G77" t="n">
-        <v>-80.83499999999999</v>
+        <v>-80.8355</v>
       </c>
       <c r="H77" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I77" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="J77" t="inlineStr">
         <is>
@@ -5754,44 +5746,48 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>07:52:00</t>
+          <t>09:20:00</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>70-80F, Medium Wind, No Rain</t>
+          <t>80-90F, Breezy</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>Long Key State Park</t>
+          <t>Martin County IRL</t>
         </is>
       </c>
       <c r="F78" t="n">
-        <v>24.80772</v>
+        <v>27.17168</v>
       </c>
       <c r="G78" t="n">
-        <v>-80.8355</v>
+        <v>-80.1833</v>
       </c>
       <c r="H78" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I78" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="J78" t="inlineStr">
         <is>
-          <t>Janice Duquesnel, Becky Collins, Mark Lee, Susan Kolterman</t>
+          <t>Ricardo Zambrano, Andrea Pereyra, Dan O'Malley</t>
         </is>
       </c>
       <c r="K78" t="inlineStr">
         <is>
-          <t>Janice.Duquesnel@dep.state.fl.us</t>
+          <t>Ricardo.Zambrano@myfwc.com</t>
         </is>
       </c>
       <c r="L78" t="inlineStr"/>
       <c r="M78" t="inlineStr"/>
-      <c r="N78" t="inlineStr"/>
+      <c r="N78" t="inlineStr">
+        <is>
+          <t>FO/OG:M/-</t>
+        </is>
+      </c>
       <c r="O78" t="inlineStr"/>
       <c r="P78" t="inlineStr">
         <is>
@@ -5855,11 +5851,7 @@
       </c>
       <c r="L79" t="inlineStr"/>
       <c r="M79" t="inlineStr"/>
-      <c r="N79" t="inlineStr">
-        <is>
-          <t>Left leg: Orange flag, upper yellow band, lower green band. Right leg: Upper silver USFWS band, lower Yellow band</t>
-        </is>
-      </c>
+      <c r="N79" t="inlineStr"/>
       <c r="O79" t="inlineStr"/>
       <c r="P79" t="inlineStr">
         <is>
@@ -5882,28 +5874,28 @@
         <v>79</v>
       </c>
       <c r="B80" s="2" t="n">
-        <v>43137</v>
+        <v>43138</v>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>09:20:00</t>
+          <t>09:15:00</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>80-90F, Breezy</t>
+          <t>60-70F, Calm, No Rain</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>Martin County IRL</t>
+          <t>Morgan Bay/Cape Romano</t>
         </is>
       </c>
       <c r="F80" t="n">
-        <v>27.17168</v>
+        <v>25.85589</v>
       </c>
       <c r="G80" t="n">
-        <v>-80.1833</v>
+        <v>-81.68340000000001</v>
       </c>
       <c r="H80" t="n">
         <v>1</v>
@@ -5913,17 +5905,21 @@
       </c>
       <c r="J80" t="inlineStr">
         <is>
-          <t>Ricardo Zambrano, Andrea Pereyra, Dan O'Malley</t>
+          <t>Kim Savides</t>
         </is>
       </c>
       <c r="K80" t="inlineStr">
         <is>
-          <t>Ricardo.Zambrano@myfwc.com</t>
+          <t>kim.savides@gmail.com</t>
         </is>
       </c>
       <c r="L80" t="inlineStr"/>
       <c r="M80" t="inlineStr"/>
-      <c r="N80" t="inlineStr"/>
+      <c r="N80" t="inlineStr">
+        <is>
+          <t>fY(20E),BO:X,Rb</t>
+        </is>
+      </c>
       <c r="O80" t="inlineStr"/>
       <c r="P80" t="inlineStr">
         <is>
@@ -5989,7 +5985,7 @@
       <c r="M81" t="inlineStr"/>
       <c r="N81" t="inlineStr">
         <is>
-          <t>fY(20E),BO:X,Rb continuing bird, will be batch reported at end of season.</t>
+          <t>G,-:fG(K5K)</t>
         </is>
       </c>
       <c r="O81" t="inlineStr"/>
@@ -6057,7 +6053,7 @@
       <c r="M82" t="inlineStr"/>
       <c r="N82" t="inlineStr">
         <is>
-          <t>G,-:fG(K5K),- continuing bird, will be batch reported at end of season.</t>
+          <t>X,-:fK(KT)</t>
         </is>
       </c>
       <c r="O82" t="inlineStr"/>
@@ -6125,7 +6121,7 @@
       <c r="M83" t="inlineStr"/>
       <c r="N83" t="inlineStr">
         <is>
-          <t>X,-:fK(KT),- continuing bird, will be batch reported at end of season.</t>
+          <t>X,O/R:O(B.),R(125)</t>
         </is>
       </c>
       <c r="O83" t="inlineStr"/>
@@ -6177,7 +6173,7 @@
         <v>1</v>
       </c>
       <c r="I84" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="J84" t="inlineStr">
         <is>
@@ -6191,11 +6187,7 @@
       </c>
       <c r="L84" t="inlineStr"/>
       <c r="M84" t="inlineStr"/>
-      <c r="N84" t="inlineStr">
-        <is>
-          <t>X,O/R:O(B.),R(125) reported to Great Lakes Plover coordinators</t>
-        </is>
-      </c>
+      <c r="N84" t="inlineStr"/>
       <c r="O84" t="inlineStr"/>
       <c r="P84" t="inlineStr">
         <is>
@@ -6218,43 +6210,39 @@
         <v>84</v>
       </c>
       <c r="B85" s="2" t="n">
-        <v>43138</v>
+        <v>43139</v>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>09:15:00</t>
-        </is>
-      </c>
-      <c r="D85" t="inlineStr">
-        <is>
-          <t>60-70F, Calm, No Rain</t>
-        </is>
-      </c>
+          <t>08:29:00</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr"/>
       <c r="E85" t="inlineStr">
         <is>
-          <t>Morgan Bay/Cape Romano</t>
+          <t>N. Hutchinson Island (north of John Brooks Beachside Park)</t>
         </is>
       </c>
       <c r="F85" t="n">
-        <v>25.85589</v>
+        <v>27.43161</v>
       </c>
       <c r="G85" t="n">
-        <v>-81.68340000000001</v>
+        <v>-80.27630000000001</v>
       </c>
       <c r="H85" t="n">
         <v>1</v>
       </c>
       <c r="I85" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="J85" t="inlineStr">
         <is>
-          <t>Kim Savides</t>
+          <t>Tim Towles</t>
         </is>
       </c>
       <c r="K85" t="inlineStr">
         <is>
-          <t>kim.savides@gmail.com</t>
+          <t>Tim.Towles@myFWC.com</t>
         </is>
       </c>
       <c r="L85" t="inlineStr"/>
@@ -6296,16 +6284,16 @@
         </is>
       </c>
       <c r="F86" t="n">
-        <v>27.43161</v>
+        <v>27.43255</v>
       </c>
       <c r="G86" t="n">
-        <v>-80.27630000000001</v>
+        <v>-80.27670000000001</v>
       </c>
       <c r="H86" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I86" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J86" t="inlineStr">
         <is>
@@ -6319,7 +6307,11 @@
       </c>
       <c r="L86" t="inlineStr"/>
       <c r="M86" t="inlineStr"/>
-      <c r="N86" t="inlineStr"/>
+      <c r="N86" t="inlineStr">
+        <is>
+          <t>FG(NLP)/-:B/M</t>
+        </is>
+      </c>
       <c r="O86" t="inlineStr"/>
       <c r="P86" t="inlineStr">
         <is>
@@ -6342,46 +6334,50 @@
         <v>86</v>
       </c>
       <c r="B87" s="2" t="n">
-        <v>43139</v>
+        <v>43137</v>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>08:29:00</t>
-        </is>
-      </c>
-      <c r="D87" t="inlineStr"/>
+          <t>13:30:00</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>70-80F, Medium Wind, No Rain</t>
+        </is>
+      </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>N. Hutchinson Island (north of John Brooks Beachside Park)</t>
+          <t>Navarre Beach Sound Side</t>
         </is>
       </c>
       <c r="F87" t="n">
-        <v>27.43255</v>
+        <v>30.3858</v>
       </c>
       <c r="G87" t="n">
-        <v>-80.27670000000001</v>
+        <v>-86.8536</v>
       </c>
       <c r="H87" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I87" t="n">
         <v>1</v>
       </c>
       <c r="J87" t="inlineStr">
         <is>
-          <t>Tim Towles</t>
+          <t>Caroline Stahala</t>
         </is>
       </c>
       <c r="K87" t="inlineStr">
         <is>
-          <t>Tim.Towles@myFWC.com</t>
+          <t>cstahala@audubon.org</t>
         </is>
       </c>
       <c r="L87" t="inlineStr"/>
       <c r="M87" t="inlineStr"/>
       <c r="N87" t="inlineStr">
         <is>
-          <t>left-- green flag NLP, right-- blue band</t>
+          <t>M/W:FY/N</t>
         </is>
       </c>
       <c r="O87" t="inlineStr"/>
@@ -6406,53 +6402,57 @@
         <v>87</v>
       </c>
       <c r="B88" s="2" t="n">
-        <v>43137</v>
+        <v>43134</v>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>13:30:00</t>
+          <t>10:30:00</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>70-80F, Medium Wind, No Rain</t>
+          <t>60-70F, Medium Wind, No Rain</t>
         </is>
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>Navarre Beach Sound Side</t>
+          <t>Outback Key</t>
         </is>
       </c>
       <c r="F88" t="n">
-        <v>30.3858</v>
+        <v>27.6495</v>
       </c>
       <c r="G88" t="n">
-        <v>-86.8536</v>
+        <v>-82.7501</v>
       </c>
       <c r="H88" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I88" t="n">
         <v>1</v>
       </c>
       <c r="J88" t="inlineStr">
         <is>
-          <t>Caroline Stahala</t>
+          <t>P.Plage, M. Parks, E. Plage L. Margeson, D. Margeson</t>
         </is>
       </c>
       <c r="K88" t="inlineStr">
         <is>
-          <t>cstahala@audubon.org</t>
+          <t>peter_plage@fws.gov</t>
         </is>
       </c>
       <c r="L88" t="inlineStr"/>
       <c r="M88" t="inlineStr"/>
       <c r="N88" t="inlineStr">
         <is>
-          <t>Silver band//white : yellow flag//black</t>
-        </is>
-      </c>
-      <c r="O88" t="inlineStr"/>
+          <t>-, O : S, Y-O</t>
+        </is>
+      </c>
+      <c r="O88" t="inlineStr">
+        <is>
+          <t>Revision. Please delete the earlier entry for Outback Key.</t>
+        </is>
+      </c>
       <c r="P88" t="inlineStr">
         <is>
           <t>WinterBirdSurvey</t>
@@ -6501,7 +6501,7 @@
         <v>2</v>
       </c>
       <c r="I89" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="J89" t="inlineStr">
         <is>
@@ -6515,11 +6515,7 @@
       </c>
       <c r="L89" t="inlineStr"/>
       <c r="M89" t="inlineStr"/>
-      <c r="N89" t="inlineStr">
-        <is>
-          <t>-, O : S, Y-O split band Reported to Great Lakes researchers</t>
-        </is>
-      </c>
+      <c r="N89" t="inlineStr"/>
       <c r="O89" t="inlineStr">
         <is>
           <t>Revision. Please delete the earlier entry for Outback Key.</t>
@@ -6550,7 +6546,7 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>10:30:00</t>
+          <t>08:15:00</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
@@ -6560,24 +6556,24 @@
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>Outback Key</t>
+          <t>Shell Key Preserve</t>
         </is>
       </c>
       <c r="F90" t="n">
-        <v>27.6495</v>
+        <v>27.6559</v>
       </c>
       <c r="G90" t="n">
-        <v>-82.7501</v>
+        <v>-82.7393</v>
       </c>
       <c r="H90" t="n">
         <v>2</v>
       </c>
       <c r="I90" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="J90" t="inlineStr">
         <is>
-          <t>P.Plage, M. Parks, E. Plage L. Margeson, D. Margeson</t>
+          <t>Peter Plage, Morgan Parks, Eric Plage, Lorraine Margeson, Don Margeson</t>
         </is>
       </c>
       <c r="K90" t="inlineStr">
@@ -6587,10 +6583,14 @@
       </c>
       <c r="L90" t="inlineStr"/>
       <c r="M90" t="inlineStr"/>
-      <c r="N90" t="inlineStr"/>
+      <c r="N90" t="inlineStr">
+        <is>
+          <t>M/BO:O/B</t>
+        </is>
+      </c>
       <c r="O90" t="inlineStr">
         <is>
-          <t>Revision. Please delete the earlier entry for Outback Key.</t>
+          <t>Surveyed Sand Key spit and nearby flats first at very low tide and returned later to count concentrated birds at mid tide. Totals reflect higher count.</t>
         </is>
       </c>
       <c r="P90" t="inlineStr">
@@ -6655,11 +6655,7 @@
       </c>
       <c r="L91" t="inlineStr"/>
       <c r="M91" t="inlineStr"/>
-      <c r="N91" t="inlineStr">
-        <is>
-          <t>S, B-O split : O, B Reported to Great Lakes researcher</t>
-        </is>
-      </c>
+      <c r="N91" t="inlineStr"/>
       <c r="O91" t="inlineStr">
         <is>
           <t>Surveyed Sand Key spit and nearby flats first at very low tide and returned later to count concentrated birds at mid tide. Totals reflect higher count.</t>
@@ -6704,13 +6700,13 @@
         </is>
       </c>
       <c r="F92" t="n">
-        <v>27.6559</v>
+        <v>27.6501</v>
       </c>
       <c r="G92" t="n">
-        <v>-82.7393</v>
+        <v>-82.7347</v>
       </c>
       <c r="H92" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I92" t="n">
         <v>1</v>
@@ -6727,7 +6723,11 @@
       </c>
       <c r="L92" t="inlineStr"/>
       <c r="M92" t="inlineStr"/>
-      <c r="N92" t="inlineStr"/>
+      <c r="N92" t="inlineStr">
+        <is>
+          <t>S, K : FO, B/Y FTP</t>
+        </is>
+      </c>
       <c r="O92" t="inlineStr">
         <is>
           <t>Surveyed Sand Key spit and nearby flats first at very low tide and returned later to count concentrated birds at mid tide. Totals reflect higher count.</t>
@@ -6781,7 +6781,7 @@
         <v>3</v>
       </c>
       <c r="I93" t="n">
-        <v>1</v>
+        <v>14</v>
       </c>
       <c r="J93" t="inlineStr">
         <is>
@@ -6795,11 +6795,7 @@
       </c>
       <c r="L93" t="inlineStr"/>
       <c r="M93" t="inlineStr"/>
-      <c r="N93" t="inlineStr">
-        <is>
-          <t>S, K : FO, B/Y FTP; Y; FTP, - : -, - reported to Great Lakes area researchers</t>
-        </is>
-      </c>
+      <c r="N93" t="inlineStr"/>
       <c r="O93" t="inlineStr">
         <is>
           <t>Surveyed Sand Key spit and nearby flats first at very low tide and returned later to count concentrated birds at mid tide. Totals reflect higher count.</t>
@@ -6826,7 +6822,7 @@
         <v>93</v>
       </c>
       <c r="B94" s="2" t="n">
-        <v>43134</v>
+        <v>43138</v>
       </c>
       <c r="C94" t="inlineStr">
         <is>
@@ -6840,39 +6836,39 @@
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>Shell Key Preserve</t>
+          <t>St Vincent NWR</t>
         </is>
       </c>
       <c r="F94" t="n">
-        <v>27.6501</v>
+        <v>29.63802</v>
       </c>
       <c r="G94" t="n">
-        <v>-82.7347</v>
+        <v>-85.148</v>
       </c>
       <c r="H94" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="I94" t="n">
-        <v>14</v>
+        <v>1</v>
       </c>
       <c r="J94" t="inlineStr">
         <is>
-          <t>Peter Plage, Morgan Parks, Eric Plage, Lorraine Margeson, Don Margeson</t>
+          <t>John Murphy</t>
         </is>
       </c>
       <c r="K94" t="inlineStr">
         <is>
-          <t>peter_plage@fws.gov</t>
+          <t>southmoonunder@mchsi.com</t>
         </is>
       </c>
       <c r="L94" t="inlineStr"/>
       <c r="M94" t="inlineStr"/>
-      <c r="N94" t="inlineStr"/>
-      <c r="O94" t="inlineStr">
-        <is>
-          <t>Surveyed Sand Key spit and nearby flats first at very low tide and returned later to count concentrated birds at mid tide. Totals reflect higher count.</t>
-        </is>
-      </c>
+      <c r="N94" t="inlineStr">
+        <is>
+          <t>S//x:YF(622)//x</t>
+        </is>
+      </c>
+      <c r="O94" t="inlineStr"/>
       <c r="P94" t="inlineStr">
         <is>
           <t>WinterBirdSurvey</t>
@@ -6935,11 +6931,7 @@
       </c>
       <c r="L95" t="inlineStr"/>
       <c r="M95" t="inlineStr"/>
-      <c r="N95" t="inlineStr">
-        <is>
-          <t>S//x:YF(622)//x</t>
-        </is>
-      </c>
+      <c r="N95" t="inlineStr"/>
       <c r="O95" t="inlineStr"/>
       <c r="P95" t="inlineStr">
         <is>
@@ -6966,44 +6958,48 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>08:15:00</t>
+          <t>09:18:00</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>60-70F, Medium Wind, No Rain</t>
+          <t>60-70F, Calm, No Rain</t>
         </is>
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>St Vincent NWR</t>
+          <t>St. George State Park</t>
         </is>
       </c>
       <c r="F96" t="n">
-        <v>29.63802</v>
+        <v>29.71343</v>
       </c>
       <c r="G96" t="n">
-        <v>-85.148</v>
+        <v>-84.7499</v>
       </c>
       <c r="H96" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="I96" t="n">
         <v>1</v>
       </c>
       <c r="J96" t="inlineStr">
         <is>
-          <t>John Murphy</t>
+          <t>Caity Reiland-Smith, Molly Tuma</t>
         </is>
       </c>
       <c r="K96" t="inlineStr">
         <is>
-          <t>southmoonunder@mchsi.com</t>
+          <t>Caity.reiland-smith@myfwc.com</t>
         </is>
       </c>
       <c r="L96" t="inlineStr"/>
       <c r="M96" t="inlineStr"/>
-      <c r="N96" t="inlineStr"/>
+      <c r="N96" t="inlineStr">
+        <is>
+          <t>YF(A41)//WK:S//BO</t>
+        </is>
+      </c>
       <c r="O96" t="inlineStr"/>
       <c r="P96" t="inlineStr">
         <is>
@@ -7044,13 +7040,13 @@
         </is>
       </c>
       <c r="F97" t="n">
-        <v>29.71343</v>
+        <v>29.71624</v>
       </c>
       <c r="G97" t="n">
-        <v>-84.7499</v>
+        <v>-84.7466</v>
       </c>
       <c r="H97" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="I97" t="n">
         <v>1</v>
@@ -7067,11 +7063,7 @@
       </c>
       <c r="L97" t="inlineStr"/>
       <c r="M97" t="inlineStr"/>
-      <c r="N97" t="inlineStr">
-        <is>
-          <t>YF(A41)//WK:S//BO</t>
-        </is>
-      </c>
+      <c r="N97" t="inlineStr"/>
       <c r="O97" t="inlineStr"/>
       <c r="P97" t="inlineStr">
         <is>
@@ -7112,13 +7104,13 @@
         </is>
       </c>
       <c r="F98" t="n">
-        <v>29.71624</v>
+        <v>29.71831</v>
       </c>
       <c r="G98" t="n">
-        <v>-84.7466</v>
+        <v>-84.744</v>
       </c>
       <c r="H98" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I98" t="n">
         <v>1</v>
@@ -7135,7 +7127,11 @@
       </c>
       <c r="L98" t="inlineStr"/>
       <c r="M98" t="inlineStr"/>
-      <c r="N98" t="inlineStr"/>
+      <c r="N98" t="inlineStr">
+        <is>
+          <t>YF(59R)//KO:S//YW</t>
+        </is>
+      </c>
       <c r="O98" t="inlineStr"/>
       <c r="P98" t="inlineStr">
         <is>
@@ -7176,13 +7172,13 @@
         </is>
       </c>
       <c r="F99" t="n">
-        <v>29.71831</v>
+        <v>29.73627</v>
       </c>
       <c r="G99" t="n">
-        <v>-84.744</v>
+        <v>-84.7229</v>
       </c>
       <c r="H99" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="I99" t="n">
         <v>1</v>
@@ -7201,7 +7197,7 @@
       <c r="M99" t="inlineStr"/>
       <c r="N99" t="inlineStr">
         <is>
-          <t>YF(59R)//KO:S//YW</t>
+          <t>S//GR:YF(C00)//WK</t>
         </is>
       </c>
       <c r="O99" t="inlineStr"/>
@@ -7244,13 +7240,13 @@
         </is>
       </c>
       <c r="F100" t="n">
-        <v>29.73627</v>
+        <v>29.7464</v>
       </c>
       <c r="G100" t="n">
-        <v>-84.7229</v>
+        <v>-84.7123</v>
       </c>
       <c r="H100" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="I100" t="n">
         <v>1</v>
@@ -7269,7 +7265,7 @@
       <c r="M100" t="inlineStr"/>
       <c r="N100" t="inlineStr">
         <is>
-          <t>S//GR:YF(C00)//WK</t>
+          <t>YO:GF//WY</t>
         </is>
       </c>
       <c r="O100" t="inlineStr"/>
@@ -7337,7 +7333,7 @@
       <c r="M101" t="inlineStr"/>
       <c r="N101" t="inlineStr">
         <is>
-          <t>YO:GF//WY</t>
+          <t>KF//R:S//YO</t>
         </is>
       </c>
       <c r="O101" t="inlineStr"/>
@@ -7403,11 +7399,7 @@
       </c>
       <c r="L102" t="inlineStr"/>
       <c r="M102" t="inlineStr"/>
-      <c r="N102" t="inlineStr">
-        <is>
-          <t>KF//R:S//YO</t>
-        </is>
-      </c>
+      <c r="N102" t="inlineStr"/>
       <c r="O102" t="inlineStr"/>
       <c r="P102" t="inlineStr">
         <is>
@@ -7430,11 +7422,11 @@
         <v>102</v>
       </c>
       <c r="B103" s="2" t="n">
-        <v>43138</v>
+        <v>43133</v>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>09:18:00</t>
+          <t>10:00:00</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
@@ -7444,29 +7436,29 @@
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t>St. George State Park</t>
+          <t>Three Rooker North Island</t>
         </is>
       </c>
       <c r="F103" t="n">
-        <v>29.7464</v>
+        <v>28.13208</v>
       </c>
       <c r="G103" t="n">
-        <v>-84.7123</v>
+        <v>-82.8282</v>
       </c>
       <c r="H103" t="n">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="I103" t="n">
         <v>1</v>
       </c>
       <c r="J103" t="inlineStr">
         <is>
-          <t>Caity Reiland-Smith, Molly Tuma</t>
+          <t>Dana Kerstein, Wendy Lichty</t>
         </is>
       </c>
       <c r="K103" t="inlineStr">
         <is>
-          <t>Caity.reiland-smith@myfwc.com</t>
+          <t>dana.kerstein@gmail.com</t>
         </is>
       </c>
       <c r="L103" t="inlineStr"/>
@@ -7498,44 +7490,48 @@
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>10:00:00</t>
+          <t>09:30:00</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>60-70F, Calm, No Rain</t>
+          <t>50-60F, Calm, No Rain</t>
         </is>
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t>Three Rooker North Island</t>
+          <t>Three Rooker South Island</t>
         </is>
       </c>
       <c r="F104" t="n">
-        <v>28.13208</v>
+        <v>28.11171</v>
       </c>
       <c r="G104" t="n">
-        <v>-82.8282</v>
+        <v>-82.837</v>
       </c>
       <c r="H104" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I104" t="n">
         <v>1</v>
       </c>
       <c r="J104" t="inlineStr">
         <is>
-          <t>Dana Kerstein, Wendy Lichty</t>
+          <t>Bob Lane, Denise Lane, Jane Mann, Steve Mann</t>
         </is>
       </c>
       <c r="K104" t="inlineStr">
         <is>
-          <t>dana.kerstein@gmail.com</t>
+          <t>Bob Lane ohiomagpie@hotmail.com</t>
         </is>
       </c>
       <c r="L104" t="inlineStr"/>
       <c r="M104" t="inlineStr"/>
-      <c r="N104" t="inlineStr"/>
+      <c r="N104" t="inlineStr">
+        <is>
+          <t>LL=S,Y RL=O,Y</t>
+        </is>
+      </c>
       <c r="O104" t="inlineStr"/>
       <c r="P104" t="inlineStr">
         <is>
@@ -7601,7 +7597,7 @@
       <c r="M105" t="inlineStr"/>
       <c r="N105" t="inlineStr">
         <is>
-          <t>LL=S,Y RL=O,Y</t>
+          <t>LL=Lb,G/R RL=S,K/W</t>
         </is>
       </c>
       <c r="O105" t="inlineStr"/>
@@ -7669,7 +7665,7 @@
       <c r="M106" t="inlineStr"/>
       <c r="N106" t="inlineStr">
         <is>
-          <t>LL=Lb,G/R RL=S,K/W</t>
+          <t>LL=FG,_ RL=S,G/G</t>
         </is>
       </c>
       <c r="O106" t="inlineStr"/>
@@ -7737,7 +7733,7 @@
       <c r="M107" t="inlineStr"/>
       <c r="N107" t="inlineStr">
         <is>
-          <t>LL=FG,_ RL=S,G/G</t>
+          <t>LL=S,_ RL=FK,_</t>
         </is>
       </c>
       <c r="O107" t="inlineStr"/>
@@ -7805,7 +7801,7 @@
       <c r="M108" t="inlineStr"/>
       <c r="N108" t="inlineStr">
         <is>
-          <t>LL=S,_ RL=FK,_</t>
+          <t>LL=FO,Y/Y RL=S,K</t>
         </is>
       </c>
       <c r="O108" t="inlineStr"/>
@@ -7873,7 +7869,7 @@
       <c r="M109" t="inlineStr"/>
       <c r="N109" t="inlineStr">
         <is>
-          <t>LL=FO,Y/Y RL=S,K</t>
+          <t>TY5 LL=FY,_ RL=S,_</t>
         </is>
       </c>
       <c r="O109" t="inlineStr"/>
@@ -7941,7 +7937,7 @@
       <c r="M110" t="inlineStr"/>
       <c r="N110" t="inlineStr">
         <is>
-          <t>TY5 LL=FY,_ RL=S,_</t>
+          <t>LL=FY,B/R RL=S,O/B</t>
         </is>
       </c>
       <c r="O110" t="inlineStr"/>
@@ -7993,7 +7989,7 @@
         <v>2</v>
       </c>
       <c r="I111" t="n">
-        <v>1</v>
+        <v>22</v>
       </c>
       <c r="J111" t="inlineStr">
         <is>
@@ -8007,11 +8003,7 @@
       </c>
       <c r="L111" t="inlineStr"/>
       <c r="M111" t="inlineStr"/>
-      <c r="N111" t="inlineStr">
-        <is>
-          <t>LL=FY,B/R RL=S,O/B</t>
-        </is>
-      </c>
+      <c r="N111" t="inlineStr"/>
       <c r="O111" t="inlineStr"/>
       <c r="P111" t="inlineStr">
         <is>
@@ -8038,45 +8030,53 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>09:30:00</t>
+          <t>08:28:00</t>
         </is>
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>50-60F, Calm, No Rain</t>
+          <t>50-60F, Breezy, No Rain</t>
         </is>
       </c>
       <c r="E112" t="inlineStr">
         <is>
-          <t>Three Rooker South Island</t>
+          <t>Tyndall Shell</t>
         </is>
       </c>
       <c r="F112" t="n">
-        <v>28.11171</v>
+        <v>30.06609</v>
       </c>
       <c r="G112" t="n">
-        <v>-82.837</v>
+        <v>-85.6161</v>
       </c>
       <c r="H112" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I112" t="n">
-        <v>22</v>
+        <v>1</v>
       </c>
       <c r="J112" t="inlineStr">
         <is>
-          <t>Bob Lane, Denise Lane, Jane Mann, Steve Mann</t>
+          <t>Marvin Friel</t>
         </is>
       </c>
       <c r="K112" t="inlineStr">
         <is>
-          <t>Bob Lane ohiomagpie@hotmail.com</t>
+          <t>marvin.friel@myfwc.com</t>
         </is>
       </c>
       <c r="L112" t="inlineStr"/>
       <c r="M112" t="inlineStr"/>
-      <c r="N112" t="inlineStr"/>
-      <c r="O112" t="inlineStr"/>
+      <c r="N112" t="inlineStr">
+        <is>
+          <t>Of//BB:S//Y</t>
+        </is>
+      </c>
+      <c r="O112" t="inlineStr">
+        <is>
+          <t>End time: 1154</t>
+        </is>
+      </c>
       <c r="P112" t="inlineStr">
         <is>
           <t>WinterBirdSurvey</t>
@@ -8141,7 +8141,7 @@
       <c r="M113" t="inlineStr"/>
       <c r="N113" t="inlineStr">
         <is>
-          <t>Of//BB:S//Y</t>
+          <t>O(blue dot)//Y:S//Y/O</t>
         </is>
       </c>
       <c r="O113" t="inlineStr">
@@ -8213,7 +8213,7 @@
       <c r="M114" t="inlineStr"/>
       <c r="N114" t="inlineStr">
         <is>
-          <t>O(blue dot)//Y:S//Y/O</t>
+          <t>O//b:S//</t>
         </is>
       </c>
       <c r="O114" t="inlineStr">
@@ -8285,7 +8285,7 @@
       <c r="M115" t="inlineStr"/>
       <c r="N115" t="inlineStr">
         <is>
-          <t>O//b:S//(missing band light blue, LR )</t>
+          <t>S//KY:Yf(H67)//W</t>
         </is>
       </c>
       <c r="O115" t="inlineStr">
@@ -8355,11 +8355,7 @@
       </c>
       <c r="L116" t="inlineStr"/>
       <c r="M116" t="inlineStr"/>
-      <c r="N116" t="inlineStr">
-        <is>
-          <t>S//KY:Yf(H67)//W (missing band Red, LR)</t>
-        </is>
-      </c>
+      <c r="N116" t="inlineStr"/>
       <c r="O116" t="inlineStr">
         <is>
           <t>End time: 1154</t>
@@ -8404,13 +8400,13 @@
         </is>
       </c>
       <c r="F117" t="n">
-        <v>30.06609</v>
+        <v>30.08727</v>
       </c>
       <c r="G117" t="n">
-        <v>-85.6161</v>
+        <v>-85.6602</v>
       </c>
       <c r="H117" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="I117" t="n">
         <v>1</v>
@@ -8427,7 +8423,11 @@
       </c>
       <c r="L117" t="inlineStr"/>
       <c r="M117" t="inlineStr"/>
-      <c r="N117" t="inlineStr"/>
+      <c r="N117" t="inlineStr">
+        <is>
+          <t>X//OG:Gf//KY</t>
+        </is>
+      </c>
       <c r="O117" t="inlineStr">
         <is>
           <t>End time: 1154</t>
@@ -8497,7 +8497,7 @@
       <c r="M118" t="inlineStr"/>
       <c r="N118" t="inlineStr">
         <is>
-          <t>X//OG:Gf//KY</t>
+          <t>Yf(82A)//WB:S//OY</t>
         </is>
       </c>
       <c r="O118" t="inlineStr">
@@ -8526,55 +8526,51 @@
         <v>118</v>
       </c>
       <c r="B119" s="2" t="n">
-        <v>43133</v>
+        <v>43137</v>
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>08:28:00</t>
+          <t>07:00:00</t>
         </is>
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>50-60F, Breezy, No Rain</t>
+          <t>60-70F, Medium Wind, No Rain</t>
         </is>
       </c>
       <c r="E119" t="inlineStr">
         <is>
-          <t>Tyndall Shell</t>
+          <t>Volusia County Atlantic Coast, Flagler County Line to north side of Ponce Inlet</t>
         </is>
       </c>
       <c r="F119" t="n">
-        <v>30.08727</v>
+        <v>29.30722</v>
       </c>
       <c r="G119" t="n">
-        <v>-85.6602</v>
+        <v>-81.0467</v>
       </c>
       <c r="H119" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="I119" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J119" t="inlineStr">
         <is>
-          <t>Marvin Friel</t>
+          <t>David Hartgrove, Rachel Ramsey, Joan Tague</t>
         </is>
       </c>
       <c r="K119" t="inlineStr">
         <is>
-          <t>marvin.friel@myfwc.com</t>
+          <t>birdman9@earthlink.net</t>
         </is>
       </c>
       <c r="L119" t="inlineStr"/>
       <c r="M119" t="inlineStr"/>
-      <c r="N119" t="inlineStr">
-        <is>
-          <t>Yf(82A)//WB:S//OY</t>
-        </is>
-      </c>
+      <c r="N119" t="inlineStr"/>
       <c r="O119" t="inlineStr">
         <is>
-          <t>End time: 1154</t>
+          <t>Disappointed that we saw no Red Knots. Surprised by the first ever American Avocets I've ever seen at the ocean shoreline.</t>
         </is>
       </c>
       <c r="P119" t="inlineStr">
@@ -8588,74 +8584,6 @@
         </is>
       </c>
       <c r="R119" t="inlineStr">
-        <is>
-          <t>Sheet1</t>
-        </is>
-      </c>
-    </row>
-    <row r="120">
-      <c r="A120" t="n">
-        <v>119</v>
-      </c>
-      <c r="B120" s="2" t="n">
-        <v>43137</v>
-      </c>
-      <c r="C120" t="inlineStr">
-        <is>
-          <t>07:00:00</t>
-        </is>
-      </c>
-      <c r="D120" t="inlineStr">
-        <is>
-          <t>60-70F, Medium Wind, No Rain</t>
-        </is>
-      </c>
-      <c r="E120" t="inlineStr">
-        <is>
-          <t>Volusia County Atlantic Coast, Flagler County Line to north side of Ponce Inlet</t>
-        </is>
-      </c>
-      <c r="F120" t="n">
-        <v>29.30722</v>
-      </c>
-      <c r="G120" t="n">
-        <v>-81.0467</v>
-      </c>
-      <c r="H120" t="n">
-        <v>6</v>
-      </c>
-      <c r="I120" t="n">
-        <v>2</v>
-      </c>
-      <c r="J120" t="inlineStr">
-        <is>
-          <t>David Hartgrove, Rachel Ramsey, Joan Tague</t>
-        </is>
-      </c>
-      <c r="K120" t="inlineStr">
-        <is>
-          <t>birdman9@earthlink.net</t>
-        </is>
-      </c>
-      <c r="L120" t="inlineStr"/>
-      <c r="M120" t="inlineStr"/>
-      <c r="N120" t="inlineStr"/>
-      <c r="O120" t="inlineStr">
-        <is>
-          <t>Disappointed that we saw no Red Knots. Surprised by the first ever American Avocets I've ever seen at the ocean shoreline.</t>
-        </is>
-      </c>
-      <c r="P120" t="inlineStr">
-        <is>
-          <t>WinterBirdSurvey</t>
-        </is>
-      </c>
-      <c r="Q120" t="inlineStr">
-        <is>
-          <t>Winter Birds 2018 Band Review.xlsx</t>
-        </is>
-      </c>
-      <c r="R120" t="inlineStr">
         <is>
           <t>Sheet1</t>
         </is>
@@ -8729,7 +8657,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-05-16 17:39</t>
+          <t>2026-05-25 12:56</t>
         </is>
       </c>
     </row>
@@ -8784,7 +8712,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>119</v>
+        <v>118</v>
       </c>
     </row>
     <row r="8">
@@ -8826,7 +8754,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>119</v>
+        <v>118</v>
       </c>
     </row>
     <row r="12">

</xml_diff>